<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 08:20 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,50 @@
         </is>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -477,24 +521,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -504,24 +548,24 @@
 132</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -543,24 +587,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -570,50 +614,6 @@
 132</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>X(대통령실 공식)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://x.com/KOREA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
@@ -628,15 +628,59 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>X(대통령실 공식)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 08:27 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -500,6 +500,50 @@
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -521,24 +565,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -548,24 +592,24 @@
 132</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -587,24 +631,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -614,50 +658,6 @@
 132</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>X(대통령실 공식)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://x.com/KOREA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
@@ -672,15 +672,59 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>X(대통령실 공식)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 08:36 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -544,6 +544,50 @@
         </is>
       </c>
       <c r="C6" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -565,24 +609,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -592,24 +636,24 @@
 132</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -631,24 +675,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -658,50 +702,6 @@
 132</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>X(대통령실 공식)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://x.com/KOREA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
@@ -716,15 +716,59 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>X(대통령실 공식)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 08:53 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -588,6 +588,50 @@
         </is>
       </c>
       <c r="C8" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -609,24 +653,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -636,24 +680,24 @@
 132</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -675,24 +719,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -702,50 +746,6 @@
 132</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>X(대통령실 공식)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://x.com/KOREA</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
@@ -760,15 +760,59 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>X(대통령실 공식)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 08:58 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -452,17 +452,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -474,17 +474,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -496,17 +496,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -518,17 +518,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -562,17 +562,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -584,17 +584,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -628,10 +628,274 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -653,24 +917,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -680,24 +944,24 @@
 132</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -719,24 +983,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -746,73 +1010,73 @@
 132</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 09:06 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -716,17 +716,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -738,17 +738,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -782,17 +782,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -848,17 +848,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -892,10 +892,274 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -917,24 +1181,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -944,24 +1208,24 @@
 132</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -983,24 +1247,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -1010,73 +1274,73 @@
 132</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 09:17 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -980,17 +980,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1002,17 +1002,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1024,17 +1024,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1046,17 +1046,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1068,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1090,17 +1090,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1112,17 +1112,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1134,17 +1134,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1156,10 +1156,274 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -1181,24 +1445,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -1208,24 +1472,24 @@
 132</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -1247,24 +1511,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Facebook(jaemyunglee)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -1274,73 +1538,73 @@
 132</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 10:00 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -711,528 +711,531 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -1244,17 +1247,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1269,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1291,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1310,17 +1313,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1332,17 +1335,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1354,17 +1357,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1379,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1398,17 +1401,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1420,10 +1423,802 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -1445,24 +2240,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -1472,24 +2267,24 @@
 132</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -1511,24 +2306,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -1538,73 +2333,73 @@
 132</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 10:37 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -853,12 +853,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
@@ -921,12 +921,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1506,528 +1506,531 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -2039,17 +2042,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2061,17 +2064,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2083,17 +2086,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2105,17 +2108,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2127,17 +2130,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2149,17 +2152,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2171,17 +2174,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2196,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2215,10 +2218,802 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -2240,24 +3035,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D118" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -2267,24 +3062,24 @@
 132</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D119" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -2306,24 +3101,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D120" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -2333,73 +3128,73 @@
 132</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D123" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D124" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 13:33 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
+          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
         </is>
       </c>
     </row>
@@ -853,168 +853,168 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>서만복 지지하고 응원합니다 1시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
+          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>Sunny Lee 지랄염병하네 56분</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1070,17 +1070,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1092,83 +1092,83 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1224,106 +1224,105 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>[공명선거 할게요. 한 표 줍쇼!]
-먼저 SNS에 후보들이 올린… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1339,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1357,17 +1356,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1379,17 +1378,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1401,17 +1400,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1423,17 +1422,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1449,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1467,17 +1466,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1489,105 +1488,105 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1603,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1621,17 +1620,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -1643,195 +1642,195 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>X(@ssaribi)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://x.com/ssaribi</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>X(@ssaribi)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://x.com/ssaribi</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1847,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1865,17 +1864,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1887,105 +1886,105 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -2002,7 +2001,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2019,106 +2018,106 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>[공명선거 할게요. 한 표 줍쇼!]
 먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2134,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2152,17 +2151,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2173,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2196,17 +2195,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2217,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2244,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2262,17 +2261,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2284,17 +2283,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2306,17 +2305,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2328,17 +2327,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2350,17 +2349,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -2372,545 +2371,548 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -2922,17 +2924,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2944,17 +2946,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2966,17 +2968,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2988,17 +2990,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3010,10 +3012,890 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -3035,24 +3917,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D158" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C159" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -3062,24 +3944,24 @@
 132</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="D159" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C160" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -3101,24 +3983,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D160" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -3128,73 +4010,73 @@
 132</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="D161" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C162" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D162" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C163" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr">
+      <c r="D163" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C164" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D164" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 16:17 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D164"/>
+  <dimension ref="A1:D202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 1시간</t>
+          <t>서만복 지지하고 응원합니다 4시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -865,46 +865,46 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
-        <is>
-          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>국민의힘 대표(장동혁)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Facebook(dhjang6971)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>임선미 이재명 탄핵 12시간</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl?comment_id=1442694117881663</t>
         </is>
       </c>
     </row>
@@ -943,34 +943,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=2186915938819611</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sunny Lee 지랄염병하네 56분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
@@ -987,34 +987,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1114,17 +1114,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -1141,34 +1141,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1268,61 +1268,61 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1400,17 +1400,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1422,17 +1422,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1510,17 +1510,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -1532,61 +1532,61 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1664,17 +1664,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
         </is>
       </c>
     </row>
@@ -1686,17 +1686,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>서만복 지지하고 응원합니다 1시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -1713,58 +1713,58 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
-        <is>
-          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
@@ -1781,34 +1781,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Sunny Lee 지랄염병하네 56분</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
         </is>
       </c>
     </row>
@@ -1825,34 +1825,34 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1979,34 +1979,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2106,62 +2106,61 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>[공명선거 할게요. 한 표 줍쇼!]
-먼저 SNS에 후보들이 올린… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2177,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2200,7 +2199,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2222,7 +2221,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2239,17 +2238,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2261,17 +2260,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2287,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2310,7 +2309,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2332,7 +2331,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2349,17 +2348,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2371,61 +2370,61 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2441,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2464,7 +2463,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2486,7 +2485,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2503,17 +2502,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -2525,151 +2524,151 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2685,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2708,7 +2707,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2730,7 +2729,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2747,17 +2746,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -2769,61 +2768,61 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2839,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2862,7 +2861,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2884,7 +2883,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2901,62 +2900,62 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>[공명선거 할게요. 한 표 줍쇼!]
 먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2972,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -2995,7 +2994,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3017,7 +3016,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3034,17 +3033,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3056,17 +3055,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3082,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3105,7 +3104,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3127,7 +3126,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3144,17 +3143,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3166,17 +3165,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3188,17 +3187,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -3210,545 +3209,548 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -3760,17 +3762,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3782,17 +3784,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3804,17 +3806,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3826,17 +3828,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3848,17 +3850,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3870,17 +3872,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3892,10 +3894,846 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -3917,24 +4755,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
+      <c r="D196" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C197" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -3944,24 +4782,24 @@
 132</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="D197" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -3983,24 +4821,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr">
+      <c r="D198" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C199" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -4010,73 +4848,73 @@
 132</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr">
+      <c r="D199" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
+      <c r="D200" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C201" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
+      <c r="D201" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C202" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 18:30 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D202"/>
+  <dimension ref="A1:D240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 4시간</t>
+          <t>서만복 지지하고 응원합니다 6시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 12시간</t>
+          <t>임선미 이재명 탄핵 14시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 5시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -987,12 +987,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 7시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=4351193995144175</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
+          <t>최민희 5시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1천</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 1시간</t>
+          <t>서만복 지지하고 응원합니다 4시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1703,46 +1703,46 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
-        <is>
-          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>국민의힘 대표(장동혁)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Facebook(dhjang6971)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>임선미 이재명 탄핵 12시간</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl?comment_id=1442694117881663</t>
         </is>
       </c>
     </row>
@@ -1781,34 +1781,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=2186915938819611</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sunny Lee 지랄염병하네 56분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
@@ -1825,34 +1825,34 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -1979,34 +1979,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2106,61 +2106,61 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2238,17 +2238,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2260,17 +2260,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -2370,61 +2370,61 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2502,17 +2502,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
         </is>
       </c>
     </row>
@@ -2524,17 +2524,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>서만복 지지하고 응원합니다 1시간</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -2551,58 +2551,58 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
-        <is>
-          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+        </is>
+      </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
@@ -2619,34 +2619,34 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Sunny Lee 지랄염병하네 56분</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
         </is>
       </c>
     </row>
@@ -2663,34 +2663,34 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2790,17 +2790,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -2817,34 +2817,34 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2944,62 +2944,61 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>[공명선거 할게요. 한 표 줍쇼!]
-먼저 SNS에 후보들이 올린… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3015,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3038,7 +3037,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3060,7 +3059,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3077,17 +3076,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3099,17 +3098,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3125,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3148,7 +3147,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3170,7 +3169,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3187,17 +3186,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3209,61 +3208,61 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3279,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3302,7 +3301,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3324,7 +3323,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3341,17 +3340,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -3363,151 +3362,151 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B137" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C137" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr">
+      <c r="D137" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3523,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -3546,7 +3545,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3568,7 +3567,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3585,17 +3584,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -3607,61 +3606,61 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3677,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -3700,7 +3699,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3722,7 +3721,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3739,62 +3738,62 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C153" t="inlineStr">
         <is>
           <t>[공명선거 할게요. 한 표 줍쇼!]
 먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="D153" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3810,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3833,7 +3832,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3855,7 +3854,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3872,17 +3871,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3894,17 +3893,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3920,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3943,7 +3942,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -3965,7 +3964,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -3982,17 +3981,17 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4004,17 +4003,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4026,17 +4025,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -4048,545 +4047,548 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -4598,17 +4600,17 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4620,17 +4622,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4642,17 +4644,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4664,17 +4666,17 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4686,17 +4688,17 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4708,17 +4710,17 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4730,10 +4732,846 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr">
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -4755,24 +5593,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr">
+      <c r="D234" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C235" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -4782,24 +5620,24 @@
 132</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr">
+      <c r="D235" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr">
+      <c r="C236" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -4821,24 +5659,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr">
+      <c r="D236" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr">
+      <c r="C237" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -4848,73 +5686,73 @@
 132</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="D237" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C238" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr">
+      <c r="D238" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C239" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D239" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr">
+      <c r="D240" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 20:48 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:D278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -836,7 +836,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl</t>
         </is>
       </c>
     </row>
@@ -853,12 +853,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 6시간</t>
+          <t>서만복 지지하고 응원합니다 9시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 14시간</t>
+          <t>임선미 이재명 탄핵 17시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 5시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 7시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 7시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 9시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>최민희 5시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1천</t>
+          <t>최민희 7시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1.1천</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 4시간</t>
+          <t>서만복 지지하고 응원합니다 6시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 12시간</t>
+          <t>임선미 이재명 탄핵 14시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 5시간</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1825,12 +1825,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 7시간</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=4351193995144175</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
+          <t>최민희 5시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1천</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 1시간</t>
+          <t>서만복 지지하고 응원합니다 4시간</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2541,46 +2541,46 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
-        <is>
-          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>국민의힘 대표(장동혁)</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Facebook(dhjang6971)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>임선미 이재명 탄핵 12시간</t>
+        </is>
+      </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl?comment_id=1442694117881663</t>
         </is>
       </c>
     </row>
@@ -2619,34 +2619,34 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=2186915938819611</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Sunny Lee 지랄염병하네 56분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
@@ -2663,34 +2663,34 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2790,17 +2790,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -2817,34 +2817,34 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2944,61 +2944,61 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3015,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3076,17 +3076,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3098,17 +3098,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3186,17 +3186,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -3208,61 +3208,61 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3340,17 +3340,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
         </is>
       </c>
     </row>
@@ -3362,17 +3362,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>서만복 지지하고 응원합니다 1시간</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -3389,58 +3389,58 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
-        <is>
-          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+        </is>
+      </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
@@ -3457,34 +3457,34 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Sunny Lee 지랄염병하네 56분</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
         </is>
       </c>
     </row>
@@ -3501,34 +3501,34 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3628,17 +3628,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -3655,34 +3655,34 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3782,62 +3782,61 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>[공명선거 할게요. 한 표 줍쇼!]
-먼저 SNS에 후보들이 올린… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3853,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3876,7 +3875,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3898,7 +3897,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3915,17 +3914,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3937,17 +3936,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3963,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -3986,7 +3985,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -4008,7 +4007,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -4025,17 +4024,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4047,61 +4046,61 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4117,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -4140,7 +4139,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4162,7 +4161,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4179,17 +4178,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -4201,151 +4200,151 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B175" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C175" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr">
+      <c r="D175" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4361,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -4384,7 +4383,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -4406,7 +4405,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -4423,17 +4422,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -4445,61 +4444,61 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4515,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -4538,7 +4537,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -4560,7 +4559,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -4577,62 +4576,62 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>[공명선거 할게요. 한 표 줍쇼!]
 먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr">
+      <c r="D191" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4649,7 +4648,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -4671,7 +4670,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -4693,7 +4692,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -4710,17 +4709,17 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4732,17 +4731,17 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4758,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -4781,7 +4780,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -4803,7 +4802,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -4820,17 +4819,17 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4842,17 +4841,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4864,17 +4863,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -4886,545 +4885,548 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -5436,17 +5438,17 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5458,17 +5460,17 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5480,17 +5482,17 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5502,17 +5504,17 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5524,17 +5526,17 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5546,17 +5548,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -5568,10 +5570,846 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -5593,24 +6431,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr">
+      <c r="D272" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B235" t="inlineStr">
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr">
+      <c r="C273" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -5620,24 +6458,24 @@
 132</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr">
+      <c r="D273" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr">
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C274" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -5659,24 +6497,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr">
+      <c r="D274" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B237" t="inlineStr">
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr">
+      <c r="C275" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -5686,73 +6524,73 @@
 132</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr">
+      <c r="D275" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr">
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C238" t="inlineStr">
+      <c r="C276" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr">
+      <c r="D276" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr">
+      <c r="C277" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr">
+      <c r="D277" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr">
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr">
+      <c r="C278" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr">
+      <c r="D278" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-20 22:25 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D278"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
+          <t>백범 김구 선생의 '문화의 힘' 비전과 평화 정신의 가치를 강조</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>대통령의 당무개입 의혹을 제기한 야당의 비판에 대해 당직선거와 공직선거의 차이를 들어 반박하는 발언</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>법이 금지하는 '당무 개입'의 법적 기준과 정의를 명확히 한 해명</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
+          <t>정청래의 알콩달콩 3분 반명을 입에 올리는 자가 반명이고, 분열을 입에 올리는 자가 분열 갈라치기다. 반명분열주의를 입에 올리는 자가 실제 반명분열주의자다. 나는 통합과 개혁만 말하겠다. 네게티브 않겠다. 헐뜯고 욕하지 않겠다. 함께 가자 통합과 개혁의 길 이종남 응원합니다 1분</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid037yt3cR9kx1jFrRnUzMHz2uBeT4Ye4afy6Brh4MsCHU4SV6DJCqyG2TxPJcVUoXspl</t>
         </is>
       </c>
     </row>
@@ -853,12 +853,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 9시간</t>
+          <t>이종남 응원합니다 1분</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl?comment_id=1347471274181464</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid037yt3cR9kx1jFrRnUzMHz2uBeT4Ye4afy6Brh4MsCHU4SV6DJCqyG2TxPJcVUoXspl?comment_id=1067159995839345</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 17시간</t>
+          <t>임선미 이재명 탄핵 18시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -943,12 +943,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 7시간</t>
+          <t>Sunhee Han 이대통령 할 일 없나봐요 본인이 더 설치고 있어요 11시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=2186915938819611</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=1310028470903780</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 9시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 11시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>최민희 7시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1.1천</t>
+          <t>최민희 59분 [감사원을 '윤석열엄호원'으로 전락시켰던 유병호구속! 차근차근 끈질기게 내란청산!]</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0XgQD6QQSRwP2tXXwtqhZFeWkZtbrtLRxFw9bMDfpzXRQRwj8nsTuDgEVbvktcMjBl</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 6시간</t>
+          <t>서만복 지지하고 응원합니다 9시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0Vezz1mhpGu4FQBnadKDVdY5cZ8Uuxzfu64DbTsdtaKUzKcAJm4QV2ezRZdRxeKDWl?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 14시간</t>
+          <t>임선미 이재명 탄핵 17시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 5시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 7시간</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 7시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 9시간</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>최민희 5시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1천</t>
+          <t>최민희 7시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1.1천</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 4시간</t>
+          <t>서만복 지지하고 응원합니다 6시간</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>임선미 이재명 탄핵 12시간</t>
+          <t>임선미 이재명 탄핵 14시간</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 5시간</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2663,12 +2663,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
+          <t>이윤이 국민이 납득할 수 있는 공정한 수사와 책임 있는 국회 운영을 기대합니다. 원칙 있는 의정활동을 응원합니다 7시간</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=4351193995144175</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
+          <t>최민희 5시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 1천</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>백범 김구 선생의 '문화의 힘'을 되새기며 평화와 문화의 가치를 강조</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>서만복 지지하고 응원합니다 1시간</t>
+          <t>서만복 지지하고 응원합니다 4시간</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -3379,46 +3379,46 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
-        <is>
-          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>국민의힘 대표(장동혁)</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Facebook(dhjang6971)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>임선미 이재명 탄핵 12시간</t>
+        </is>
+      </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl?comment_id=1442694117881663</t>
         </is>
       </c>
     </row>
@@ -3457,34 +3457,34 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
+          <t>백광규 끌어들이는게 누구요..? 친명팔이들 아니오..? 2시간</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=2186915938819611</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Sunny Lee 지랄염병하네 56분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
@@ -3501,34 +3501,34 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Duckchun Ryu 하루속히 당내분을 정리하고 당이 하나되어 국민의 지지와 신뢰를 얻기를 바랍니다. 4시간</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1406297634696711</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3628,17 +3628,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -3655,34 +3655,34 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3782,61 +3782,61 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>최민희 3시간 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요!</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>백범 김구 선생의 '문화의 힘' 사상과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
+          <t>칼레드 알-아나니 유네스코 사무총장과의 면담을 통한 대한민국과 유네스코의 협력 및 발전 방향 논의</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>야당의 '대통령 당무 개입' 주장을 당직선거와 공직선거의 구분 무지로 규정하며 비판</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>공직선거법상 불법 당무개입의 법적 기준을 설명하며 자신을 향한 비판에 해명하는 글</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3914,17 +3914,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3936,17 +3936,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -4024,17 +4024,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -4046,61 +4046,61 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4178,17 +4178,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>260720_&lt;제3차 정기전국당원대회 당대표·최고위원 선출을 위한 예비경선 합동연설회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l</t>
         </is>
       </c>
     </row>
@@ -4200,17 +4200,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>서만복 지지하고 응원합니다 1시간</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464</t>
         </is>
       </c>
     </row>
@@ -4227,58 +4227,58 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+          <t>Begonia Song 서만복 국짐당 신첝ㆍ 1시간</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02ZCeAvwLB849zAoTGw7q4NJpNyQmjGAyMjCAYMkh25tin64vL489rSUwnZ5wPnWU5l?comment_id=1347471274181464&amp;reply_comment_id=899432305972041</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
-        <is>
-          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>국민의힘 대표(장동혁)</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>Facebook(dhjang6971)</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+        </is>
+      </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
@@ -4295,34 +4295,34 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
+          <t>오세득 끌어들이긴 누가 끌어들여? 지가 제발로들어와서 난동 피우는거 아니야? 2시간</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/3062093377317802/</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
+          <t>Sunny Lee 지랄염병하네 56분</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
+          <t>https://www.facebook.com/reel/3062093377317802/?comment_id=952656431213277&amp;reply_comment_id=2372600373662130</t>
         </is>
       </c>
     </row>
@@ -4339,34 +4339,34 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 3시간</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -4466,17 +4466,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -4493,34 +4493,34 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -4620,62 +4620,61 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>[공명선거 할게요. 한 표 줍쇼!]
-먼저 SNS에 후보들이 올린… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
+          <t>최민희 29분 [송영길후보, 오늘 연설 땐 안그러시더만!] 돌아서기 무섭게 "정청래대표되면 청와대가 상대안할 것"이라니, 당원님들이 후보님 상대 안하고 싶겠어요! 서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
+          <t>서무수 참 추하네요. 한때 존경하였는데. 18분</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02Z7WTwQrmVLCnHpTipWk1wvys3e2QFFwpa2cxXjkJqM3jFTtF1ibYVZnkfrCP4Laxl?comment_id=1774716837217310</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4691,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -4714,7 +4713,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -4736,7 +4735,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -4753,17 +4752,17 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>과거 대통령들의 선례를 든 누리꾼의 지적에 법이 금지하는 '당무 개입'의 법적 기준을 설명하며 해명하는 글</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4775,17 +4774,17 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4801,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -4824,7 +4823,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -4846,7 +4845,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -4863,17 +4862,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -4885,61 +4884,61 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4955,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -4978,7 +4977,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -5000,7 +4999,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -5017,17 +5016,17 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -5039,151 +5038,151 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 5시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.6천 안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>안재갑 지난번 당대표때 우리식구 싹다 당신을 찍어줬음. 당대표 한번했고 지선 망하게 했으면 책임지고 그만 하시는게 좋다고 생각함. 자꾸 그래봐야 민주당원을 갈라치는 일만하는것 같아 안타까움.. 4시간</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=917519840631017</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr">
+      <c r="B213" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
+      <c r="C213" t="inlineStr">
         <is>
           <t>이재명 대통령, 또 시작이다.
 많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
 도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr">
+      <c r="D213" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/2351791568896459/</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>국민의힘 원내대표(정점식)</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>Facebook(jsjeong0403)</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
+          <t>&lt;몰상식한 정쟁에 대통령을 끌어들이지 마십시오&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
+          <t>https://www.facebook.com/reel/3062093377317802/</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;필리버스터를 통해 민주당의 입법 폭주와 특검 연장의 모순을 국민 여러분께 낱낱이 알리겠습니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>이종원 어런 dog 같은.더불당 해체대상이다. 14분</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid0vseiUsEJ673FKpjzfGVSXDYcmSNTRvrnh91ehg5MU2FPiUrYeqXX6NhHxkZETppYl?comment_id=1747172316631031</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5199,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -5222,7 +5221,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -5244,7 +5243,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -5261,17 +5260,17 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -5283,61 +5282,61 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5353,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -5376,7 +5375,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -5398,7 +5397,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -5415,62 +5414,62 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr">
+      <c r="C229" t="inlineStr">
         <is>
           <t>[공명선거 할게요. 한 표 줍쇼!]
 먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="D229" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5486,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
+          <t>백범 김구 선생의 '문화의 힘'과 유네스코 헌장의 평화 정신을 강조</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -5509,7 +5508,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과 대한민국 간의 협력 및 발전 방향을 논의한 면담</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -5531,7 +5530,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
+          <t>당직선거와 공직선거를 구분하지 못한 채 '당무개입'이라 주장하는 야당의 비판 논평을 반박</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -5548,17 +5547,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5570,17 +5569,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5596,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -5619,7 +5618,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -5641,7 +5640,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -5658,17 +5657,17 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -5680,17 +5679,17 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -5702,17 +5701,17 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
         </is>
       </c>
     </row>
@@ -5724,545 +5723,548 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>정청래의 알콩달콩 4시간 투표도 1인1표이듯이 싸움도 1대1이었으면... 민주당다운 민주당은 제가 지킬테니 당원들께서 저를 지켜주십시오. 2.5천 Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>Dongsup Kang 김어준, 유시민 등에 업고 대통령님한테 싸움 건게 누군데! 확마! 가증스러워서 이번에 보내줄테니 곱게 가슈! 4시간</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02fcHQcchEN2U8N9e8JTH53ErLDSZUZR8wJaKsjU1NPyCYJ3FUkwFTVeyMZQeGjQhsl?comment_id=1046215424583951</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>이재명 대통령, 또 시작이다.
+많은 사람이 비판하면 스스로 한 번 돌아볼 법도 한데,
+도무지 그런 생각은 하지 않는다.… 더 보기</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0369jC6BuijYiiakZFtQvRNB3saMixqzf3wKLucA62VY5XijVYqjjBb9RZp2JFY8jnl</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>&lt;종합특검법 개정, 내란 끝까지 발본색원!&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://www.facebook.com/reel/2351791568896459/</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>&lt;국민의힘 최고위원회(7.20)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/reel/1403688621817668/</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>박순옥 장동혁대표님 함께!! 응원합니다 3시간</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/reel/1403688621817668/?comment_id=2232283440918980</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>&lt;14년 만에 다시 시작한 한몽 과학기술 협력&gt; 대통령님의 이번 몽골 국빈방문을 수행하며 울란바타르에서 여러 일정을 함께했습니다. 15년 만의 국빈방문인 만큼 양국 관계에 대한 기대가 크다는 것을 현장에서 느꼈습니다. 대통령님께서 방명록에 남기신 “우정과 신뢰 위에 한몽 황금시대를 더 보기</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid0RunEkCFt4vUoLbFDuYUECs7sWMDdLVTHtcTDR2Wqd9KmXzZd53rEvpQCqhAxf5rDl?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! v.daum.net "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 (지디넷코리아=박수형 기자)더불어민주당 최민희 의원이 국회의원도 국민소환제의 대상에 포함하는 ‘국회의원의 국민소환에 관한 법률안’을 대표발의 했다고 6일 밝혔다. 국회의원에 대한 국민의 민주적 통제 권한을 부여하고, 대의민주주의의 한계를 보완하겠다는 취지다. 지난 2006년 지방자치단체장과 지방의회 의원에 대한 주</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>[공명선거 할게요. 한 표 줍쇼!]
+먼저 SNS에 후보들이 올린… 더 보기</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0X8BdAckvZWtW2jS83D7GX9bZDJEgvc3QAWJtszQ7vmDTFZ8JYyQtxC6iAogNFBHRl</t>
         </is>
       </c>
     </row>
@@ -6274,17 +6276,17 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>백범 김구 선생은 군사나 경제적 강국보다 문화의 힘으로 인류 평화에 기여하는 나라를 지향했습니다. 그는 인간의 불행을 극복하고 진정한 평화를 실현할 열쇠가 문화에 있다고 보았습니다.</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -6296,17 +6298,17 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>부산에서 열린 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사와 향후 발전 방안을 논의했습니다.</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -6318,17 +6320,17 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>야당이 당직선거와 공직선거를 구분하지 못한 채 대통령의 행위를 불법 당무개입이라 비판하는 것에 대해, 기초적인 상식조차 결여된 잘못된 주장이라며 강하게 반박했습니다.</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -6340,17 +6342,17 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>법이 금지하는 '당무 개입'은 선거 공천이나 경선에 부당하게 관여하는 것을 의미하며, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않습니다.</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -6362,17 +6364,17 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>돈 때문에 선거에 나서지 못하는 상황은 부정부패를 유발할 수 있으므로, 노무현 전 대통령이 도입한 '돈 안 드는 선거(선거공영제)' 개혁의 가치를 이어가야 합니다.</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -6384,17 +6386,17 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>이재명 의원은 제헌절을 맞아 민주주의를 끝까지 수호하겠다는 의지를 표명했습니다.</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -6406,10 +6408,846 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>이재명 유튜브 채널을 통해 보건복지부, 식품의약품안전처 등 주요 부처의 업무보고를 진행하는 라이브 방송 '잼프의 장관들' 시즌2의 새로운 에피소드가 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 국토교통부, 농림축산식품부, 해양수산부의 업무보고를 다루는 신규 라이브 방송을 오후 1시 50분에 공개할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>7월 16일 유튜브 '잼플릭스' 채널을 통해 새로운 영상 에피소드들이 시간대별로 순차적으로 공개됩니다.</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>정부 부처들이 참여하는 '국민과 함께하는 업무보고 시즌 2'가 현재 유튜브를 통해 실시간으로 방송 중입니다.</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C272" t="inlineStr">
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>민주주의를 수호하기 위해 함께 힘써 준 국민들에게 깊은 감사의 뜻을 전하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>작성자는 해당 인물에게 바라는 유일한 요구사항은 검찰개혁뿐임을 강조하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>백범 김구 선생은 경제적 부강함보다 높은 문화의 힘으로 인류 평화에 공헌하는 나라를 지향했습니다. 그는 인간 내면의 문제를 해결하고 평화를 이룩하는 핵심 열쇠가 바로 문화에 있다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>부산 세계유산위원회에 참석한 칼레드 알-아나니 유네스코 사무총장과 만나 한국과 유네스코의 협력 역사 및 향후 발전 방향에 대해 의견을 나누었습니다.</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>작성자는 법이 금지하는 당무 개입이란 공직선거의 공천이나 경선에 관여하는 위법 행위를 의미하므로, 일상적인 당무에 의견을 제시하는 것은 이에 해당하지 않는다고 반박했습니다.</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>선거 비용 부담이 부정부패를 유발하는 문제를 해결하기 위해 도입된 노무현 전 대통령의 '돈 안 드는 선거(선거공영제)'는 한국 정치를 근본적으로 바꾼 핵심 개혁입니다.</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>이재명 대표는 제헌절을 맞아 어떤 역경 속에서도 민주주의를 굳건히 지켜내겠다는 의지를 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>이재명 의원의 유튜브 채널에서 보건복지부와 식품의약품안전처 등 주요 부처의 업무보고를 다루는 '잼프의 장관들' 시즌2 라이브 방송이 공개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>X(@KOREA)</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://x.com/KOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0oG7aNFCNrAqT5bfgT2SEecH9xCmnnjMD6iHYQ4rpCn5pXqSWMRrVpVxCrYwVirkil?comment_id=1341196558137916</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -6431,24 +7269,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
+      <c r="D310" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C311" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -6458,24 +7296,24 @@
 132</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D311" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C274" t="inlineStr">
+      <c r="C312" t="inlineStr">
         <is>
           <t>이재명
 3일
@@ -6497,24 +7335,24 @@
 답글 11개 모두 보기</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
+      <c r="D312" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr">
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
         <is>
           <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr">
+      <c r="C313" t="inlineStr">
         <is>
           <t>이계승
 난그에게,별로바라는게,없다.
@@ -6524,73 +7362,73 @@
 132</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr">
+      <c r="D313" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
         <is>
           <t>X(대통령실 공식)</t>
         </is>
       </c>
-      <c r="C276" t="inlineStr">
+      <c r="C314" t="inlineStr">
         <is>
           <t>유튜브 콘텐츠 '잼플릭스' 7월 16일 신규 에피소드 3편 공개 소식 안내</t>
         </is>
       </c>
-      <c r="D276" t="inlineStr">
+      <c r="D314" t="inlineStr">
         <is>
           <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B277" t="inlineStr">
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C277" t="inlineStr">
+      <c r="C315" t="inlineStr">
         <is>
           <t>3년 전 오늘 발생한 참사로 희생된 열네 분을 추모하는 글</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr">
+      <c r="D315" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jaemyunglee</t>
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
         <is>
           <t>X(개인)</t>
         </is>
       </c>
-      <c r="C278" t="inlineStr">
+      <c r="C316" t="inlineStr">
         <is>
           <t>형사재판의 유죄 증명 기준을 설명한 이건태 의원 글을 공유</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr">
+      <c r="D316" t="inlineStr">
         <is>
           <t>https://x.com/Jaemyung_Lee</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 03:31 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -447,66 +447,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>백범 김구 선생의 정신을 기리며 문화의 힘과 평화의 가치를 강조</t>
+          <t>&lt;이런 황당한 네거티브가 먹힐거라 생각하는가?&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid05EYb3AnuKdFVC6bxmfVdYRg1aanAG6vpT6ZcXDk4D24tXyZko5Pb3M25cV7rpp9Ul</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과의 면담 및 양측의 협력·발전 방향 논의</t>
+          <t>신성회 1분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid05EYb3AnuKdFVC6bxmfVdYRg1aanAG6vpT6ZcXDk4D24tXyZko5Pb3M25cV7rpp9Ul?comment_id=1019257851015468</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>'당무개입' 비판에 대해 불법 행위의 법적 기준과 정의를 설명하는 글</t>
+          <t>백범 김구 선생의 정신을 기리며 문화의 힘과 평화의 가치를 강조</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>노무현 전 대통령의 정치개혁 유산인 '돈 안 드는 선거(선거공영제)'의 중요성을 강조</t>
+          <t>부산 세계유산위원회에 참석한 유네스코 사무총장과의 면담 및 양측의 협력·발전 방향 논의</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -562,17 +562,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -584,17 +584,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>'당무개입' 비판에 대해 불법 행위의 법적 기준과 정의를 설명하는 글</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>노무현 전 대통령의 정치개혁 유산인 '돈 안 드는 선거(선거공영제)'의 중요성을 강조</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
@@ -694,83 +694,83 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl?comment_id=1341196558137916</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>이계승 난그에게,별로바라는게,없다. 있다면,딱,하나.검찰개혁! 3일</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl?comment_id=1341196558137916</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&lt;때만 되면 나타나는...습관성 남탓공격인가?&gt;… 더 보기</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0k5mX4cV1SaFRpBvNVKkaGjUtux1JZfS8vGPa6FGCcWLXb38AtDpBgffQacL59eaXl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
@@ -848,193 +848,193 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>김규호 응원합니다 화이팅 19분</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0k5mX4cV1SaFRpBvNVKkaGjUtux1JZfS8vGPa6FGCcWLXb38AtDpBgffQacL59eaXl?comment_id=1375061374499216</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>"자아비판중?"</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>주정빈 여지것 취임후 국가를 위해 한것 뭐있냐 31분</t>
+          <t>&lt;때만 되면 나타나는...습관성 남탓공격인가?&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl?comment_id=2274036606745491</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0k5mX4cV1SaFRpBvNVKkaGjUtux1JZfS8vGPa6FGCcWLXb38AtDpBgffQacL59eaXl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
+          <t>김규호 응원합니다 화이팅 19분</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0k5mX4cV1SaFRpBvNVKkaGjUtux1JZfS8vGPa6FGCcWLXb38AtDpBgffQacL59eaXl?comment_id=1375061374499216</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 원내대책회의(7.21)&gt;… 더 보기</t>
+          <t>"자아비판중?"</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/863734739870492/</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sky Lee Myeobg Seub 원구성도 안하구 이게 머꼬 13분</t>
+          <t>주정빈 여지것 취임후 국가를 위해 한것 뭐있냐 31분</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/863734739870492/?comment_id=1776191500070672</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl?comment_id=2274036606745491</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
+          <t>&lt;국민의힘 원내대책회의(7.21)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/863734739870492/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>Sky Lee Myeobg Seub 원구성도 안하구 이게 머꼬 13분</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/863734739870492/?comment_id=1776191500070672</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
+          <t>&lt;취임 1년 다시 미래를 생각합니다&gt; 오늘은 과학기술정보통신부 장관으로 임명된 지 꼭 1년이 되는 날입니다. 공교롭게도 오늘은 대통령께 두번째 업무보고를 드리는 날이기도 했습니다. 지난 1년을 돌아보며 앞으로 무엇을 더 준비해야 할지 다시 생각하게 되는 하루였습니다. 지난 1년 동안 가장 더 보기</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1112,83 +1112,83 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>&lt;중국의 AI 통제 움직임이 우리에게 던지는 질문&gt; 중국이 자국의 주요 AI 모델에 대한 해외 접근 제한을 검토하고 있다는 소식은 단순한 기업 정책의 변화가 아닙니다. AI가 이제 국가안보와 산업 경쟁력을 좌우하는 전략 자산이 되었음을 보여주는 중요한 신호입니다. 이미 미국은 최첨단 AI 더 보기 The Chinese AI Blockade Is Coming 보낸 사람: forbes.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>강호율 손가락만 빨고 있을 것인가, 미래를 선점할 것인가! 2주</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l?comment_id=2002800833940278</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>최민희 1시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 39분</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1266,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 39분</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl?comment_id=1375184588071436</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>[한 표는 최민희에게!!]… 더 보기</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0wVh2Eyw2HozkzFgVRvcKckRV7zgdnkt38gjdQkwocz6V3jNJAMRzaCHqgQhJqofJl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1315,10 +1315,76 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>최민희 1시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 39분</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 39분</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl?comment_id=1375184588071436</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>[한 표는 최민희에게!!]… 더 보기</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0wVh2Eyw2HozkzFgVRvcKckRV7zgdnkt38gjdQkwocz6V3jNJAMRzaCHqgQhJqofJl</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
           <t>이장주 투표했습니다. 26분</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0wVh2Eyw2HozkzFgVRvcKckRV7zgdnkt38gjdQkwocz6V3jNJAMRzaCHqgQhJqofJl?comment_id=1789603429077345</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 07:09 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,12 +453,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,12 +468,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -495,7 +495,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -603,12 +603,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -738,24 +738,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,24 +900,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 3시간 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 1.6천 Ys Lee 최민희 의원님이 해결해주실거예요 그쪽으로 잘 아심 3시간</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02e4qjXsCusP6Tr8CEFQg6hUY35wVGyLK7ryt26n3VvStk7uEgFYdFGqc3urYmQhw7l</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,24 +927,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>"자아비판중?"</t>
+          <t>정청래의 알콩달콩 3시간 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 1.6천 Ys Lee 최민희 의원님이 해결해주실거예요 그쪽으로 잘 아심 3시간</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02e4qjXsCusP6Tr8CEFQg6hUY35wVGyLK7ryt26n3VvStk7uEgFYdFGqc3urYmQhw7l</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,68 +954,68 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
+          <t>"자아비판중?"</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>이번 선관위 특검법 합의의 핵심은 “야당의 동의 없이, 특검 추천은 없다”는 것입니다.
 야당 추천위원들이 동의해줄 수 없는 추천안이 올라오면, 추천 단체에 재추천을 거듭 요구할 수 있도록 합의했습니다. 
 야당의 추천권이 보장된 국민추천특검입니다. … 더 보기</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jsjeong0403/posts/pfbid0BUgkRDVZo4TJP7J82i5vjwzjPaF8AjxpaGbi3Y63CH9eZwo136hhkVbvL7Y7AjWYl</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>과학기술정보통신부 장관 취임 1주년 소회와 미래 과학기술·ICT 정책 추진에 대한 다짐</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>과학기술정보통신부 장관 취임 1주년 소회와 미래 과학기술·ICT 정책 추진에 대한 다짐</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>중국의 AI 모델 해외 접근 제한 조치와 전략 자산으로서의 AI가 지닌 안보·산업적 시사점을 조명하는 분석</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1145,24 +1145,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>중국의 AI 모델 해외 접근 제한 조치와 전략 자산으로서의 AI가 지닌 안보·산업적 시사점을 조명하는 분석</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1307,12 +1307,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>최민희 5시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 1천 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 4시간</t>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1334,10 +1334,37 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
+          <t>최민희 5시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 1천 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 4시간</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>최민희 2시간 [김민석후보님, 신천지가 민주당 전대에 개입한 근거있다구요?깜놀 입니다. 근거를 즉시 공개하고 신천지개입을 선제차단하십시다! [적절한 시기]에 공개한다니, [지금]이 [적절한 시기]인 거 모르세요? 1천 심화섭 근거가 있음 선제적으로 문제해결을 해야지요. 쥐고 있을 이유는 없습니다. 1시간</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid02fT13wrpb8dM61CCahVNjR7LetrvTm7J1rrohDRfRk4EXhr5Evsm9hyoctwWLcxHil</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 07:44 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,66 +453,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>확인불가</t>
+          <t>6시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>최민희 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 1.1천 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>확인불가</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
+          <t>최민희 [김민석후보님, 신천지가 민주당 전대에 개입한 근거있다구요?깜놀 입니다. 근거를 즉시 공개하고 신천지개입을 선제차단하십시다! [적절한 시기]에 공개한다니, [지금]이 [적절한 시기]인 거 모르세요? 1.1천 심화섭 근거가 있음 선제적으로 문제해결을 해야지요. 쥐고 있을 이유는 없습니다.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02fT13wrpb8dM61CCahVNjR7LetrvTm7J1rrohDRfRk4EXhr5Evsm9hyoctwWLcxHil</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -522,12 +522,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:33</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
+          <t>칼레드 알-아나니 유네스코 사무총장님께서 부산에서 열리는 세계유산위원회에 참석해 주셨습니다. 우리는 그간 대한민국과 유네스코가 함께 쌓아온 협력과 앞으로의 발전 방향에 대해 뜻깊은 대화를 나눴습니다. 대한민국은 유네스코와 깊은 인연을 이어왔습니다. 6·25전쟁 직후 유네스코의 지원으로 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
+          <t>공당이 당직선거와 공직선거 조차 구분하지 못하면 안됩니다. 그건 국정과 개인사업을 구별못하는 것만큼 심각한 문제입니다. 그런 역량으로는 국정을 감당하기 어렵습니다. 비난 논평 내실때 최소한의 상식은 갖추시는게 좋겠습니다. 공직자인 당원의 당내 공직선거 관여 = 불법 당무개입이자 더 보기 뉴스1 @News1Kr 7월 19일 野 "李대통령 與 선거 기탁금 가이드라인 하달…명백한 당무개입" #뉴스1  news1.kr/politics/assem…</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -630,12 +630,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
+          <t xml:space="preserve">우선 풀잎이님의 의견과 질책은 감사하게 받아들입니다. 다만, 법이 금한 당무개입이란 공직선거법 등 법률에 위반하여 공직선거 공천이나 경선에 관여하는 경우를 말하는 것입니다. 박근혜 대통령 사례는 공직선거 후보 공천이나 경선에 개입했기 때문에 문제된 것이지 일상적 당무에 의견을 낸 더 보기 풀잎이 (풀잎이) @ip_pul93952 7월 19일 @Jaemyung_Lee 님에게 보내는 답글 지금당신이  대통령이지  민주당 당대표인지  착각하시는것같은데   당무개입으로 박근혜2년 감빵 노무현 전대통령님   당무개입도아닌데   열린우리당  </t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@KOREA)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -657,12 +657,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>돈 때문에 선거에 나갈 수 없다는 건 슬픈 일이기도 하지만, 부정부패의 유인을 키우는 일이기도 합니다. 모두가 인정하는, 그리고 대한민국의 정치를 근본적으로 바꾼 노무현 정치개혁의 핵심중 하나는 돈 안드는 선거 즉 선거공영제 도입이었습니다. 노무현 대통령님의 '돈안드는 선거' 개혁이 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/KOREA</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
+          <t>❝ 흔들리지언정 결코 무너지지 않습니다 ❞ 📎 youtube.com/shorts/UB4cgzo… #이재명 #제헌절 #빛의위원회 #민주주의 02:14</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
+          <t>잠시 뒤 새로운 에피소드 공개 잼프의 장관들 [coming soon] youtube.com [#이재명 LIVE] 🔔 맞춤 알림 : 국민주권정부는 어떻게 일하고 있을까? '잼프의 장관들' 시즌2 | 보건복지부,... 보건복지부, 식품의약품안전처, 성평등가족부, 국민권익위원회 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
+          <t>30분 뒤 새로운 에피소드 공개 맨 앞줄 장관 [13:50 공개] youtube.com [#이재명 LIVE] 오늘의 TOP 10 콘텐츠(가 될까요?) '맨 앞줄 장관' | 국토교통부, 농림축산식품부, 해양수산부... 국토교통부, 농림축산식품부, 해양수산부 업무보고 (2026. 7. 16.)#이재명 #대통령 #업무보고</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,24 +765,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
+          <t>잼플릭스 7월 16일 새로운 에피소드 공개 바쁘지만 보고는 받고 싶어 [10:00 공개] 📎 youtube.com/live/ioP47qdN2… 맨 앞줄 장관 [13:50 공개] 📎 youtube.com/live/Fpj35dsji… 잼프의 장관들 [16:10 공개] 📎 youtube.com/live/-yoxtsnZG… 🎧 팟캐스트 : youtube.com/playlist?list=…</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>X(@KOREA)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,24 +792,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
+          <t>✨국민 여러분께 추천하는 신규 콘텐츠 국민과 함께하는 업무보고 시즌2 : 보고 천국 편 절찬 스트리밍 중! 👉 지금 시청하기 : youtube.com/live/Uvw4HWEWJ… #재정경제부 #국가데이터처 #금융위원회 #기획예산처</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://x.com/KOREA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@ssaribi)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,12 +819,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
+          <t>&lt;민주주의를 지켜주신 위대한 대한국민 여러분께&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/ssaribi</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02rdbkzGYzt2ezrSbM5gNL4xGtLXMk36oHJAQfvpmroaQUEcqdNwmqrYTBtb5BMdFXl</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
+          <t>&lt;천재소녀가 나타났다.&gt; 정치신동의 탄생을 경축합니다. 무한폭풍RT로 축하해주세요!</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
+          <t>&lt;소위 문자폭탄에 대하여&gt;국회의원들은 선거철이 오면 원하지 않는 문자폭탄을 무차별적으로 보낸다. 연말 후원금 시즌이 오면 또 문자폭탄을 보낸다. 국회의원들은 문자보내도 되고 국민들은 국회의원에게 항의문자보내면 안 되나? 세상이 바뀌었다, 적응들하시길.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
+          <t>&lt;국민여러분께 부탁드립니다.&gt; 저는 문재인대통령의 개헌안을 지지합니다. 여러분들도 지지 좀 해주시겠습니까? 지지하신다면...무한폭풍RT~발사!</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,24 +927,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 3시간 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 1.6천 Ys Lee 최민희 의원님이 해결해주실거예요 그쪽으로 잘 아심 3시간</t>
+          <t>President Donald Trump, thanks to you, the spring of peace is on the Korean peninsula. Thank you. Please help us to establish peace on the Korean Peninsula in the future. The Korean people support you. Nobel Peace Prize winner ,,, Good luck with you! Donald J. Trump @realDonaldTrump 2018년 4월 27일 @re</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02e4qjXsCusP6Tr8CEFQg6hUY35wVGyLK7ryt26n3VvStk7uEgFYdFGqc3urYmQhw7l</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@ssaribi)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,24 +954,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>"자아비판중?"</t>
+          <t>&lt;가는길 험난해도 웃으며 가겠습니다&gt;초선때 조중동과의싸움-18대총선 보수언론공격 낙선-19대 서울최상위권 성적 당선-국정원과의 싸움-세월호 단식-최고위원당선-징계-컷오프-더컸유세단-가족 공격. 영광보다 고난의 길이지만 여러분과 함께 웃으며 가겠습니다</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
+          <t>https://x.com/ssaribi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,95 +981,95 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
+          <t>정청래의 알콩달콩 3시간 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 1.6천 Ys Lee 최민희 의원님이 해결해주실거예요 그쪽으로 잘 아심 3시간</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02e4qjXsCusP6Tr8CEFQg6hUY35wVGyLK7ryt26n3VvStk7uEgFYdFGqc3urYmQhw7l</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>국민의힘 대표(장동혁)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Facebook(dhjang6971)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>"자아비판중?"</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid066ZeMzTgWfzGryQVHja28BkK5r5AMw17vMr1MDyxrc1DZZhU4vmJyzqazrNuLHbxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>더불어민주당 원내대표(한병도)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Facebook(hbd7851)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/hbd7851/posts/pfbid02yA82MUpkmbFcn1HeGmtrgjdJqyRjQkS8zR8vip5VQ3Z596dkZRn9KYVFShAhi2cSl</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>이번 선관위 특검법 합의의 핵심은 “야당의 동의 없이, 특검 추천은 없다”는 것입니다.
 야당 추천위원들이 동의해줄 수 없는 추천안이 올라오면, 추천 단체에 재추천을 거듭 요구할 수 있도록 합의했습니다. 
 야당의 추천권이 보장된 국민추천특검입니다. … 더 보기</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jsjeong0403/posts/pfbid0BUgkRDVZo4TJP7J82i5vjwzjPaF8AjxpaGbi3Y63CH9eZwo136hhkVbvL7Y7AjWYl</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>과학기술정보통신부 장관 취임 1주년 소회와 미래 과학기술·ICT 정책 추진에 대한 다짐</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
+          <t>과학기술정보통신부 장관 취임 1주년 소회와 미래 과학기술·ICT 정책 추진에 대한 다짐</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>중국의 AI 모델 해외 접근 제한 조치와 전략 자산으로서의 AI가 지닌 안보·산업적 시사점을 조명하는 분석</t>
+          <t>&lt;국제물리올림피아드 금메달, 진심으로 축하합니다&gt; 출정식에서 학생들과 함께했던 시간이 아직도 생생합니다. 긴장된 표정 속에서도 과학을 향한 호기심과 자신감이 빛났고, 서로를 격려하며 세계 무대를 향해 나아가던 모습에서 대한민국 과학의 미래를 보았습니다. 그리고 그 믿음이 현실이 더 보기</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(msitminister)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1172,24 +1172,24 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
+          <t>&lt;김빛내리 단장님의 아시아 최초 나카소네상 수상을 축하합니다&gt; 국제적으로 반가운 소식을 전합니다. 김빛내리 기초과학연구원(IBS) RNA 연구단장님께서 2027년 휴먼프론티어사이언스프로그램(HFSP) 나카소네상 수상자로 선정되셨습니다. 한국인 최초이자 아시아 최초 수상입니다. 진심으로 더 보기</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1199,24 +1199,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
+          <t>중국의 AI 모델 해외 접근 제한 조치와 전략 자산으로서의 AI가 지닌 안보·산업적 시사점을 조명하는 분석</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>과방위원장(최민희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@minhee_choi_)</t>
+          <t>Facebook(msitminister)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1226,12 +1226,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
+          <t>배경훈 부총리 겸 과학기술정보통신부 장관의 SNS 계정을 안내해드립니다. 국민들과 더 가깝게 소통하겠습니다. 감사합니다.… 더 보기</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/minhee_choi_</t>
+          <t>https://www.facebook.com/msitminister/posts/pfbid02VmDwvsBhvEuHdDskewgq7VTTRY9y5P465t1qm2yKdcw5KvbXacfRoB7zR33zXSN1l</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
+          <t>[트친님들의 10만원을 언론개혁ㆍ정치개혁의 밑거름으로!] 비례대표 국회의원 시절 저는 후원회를 열지 않았습니다. 필요가 없었기 때문입니다. 지역구 국회의원을 처음 해보는데요, 지역구 운영비가 생각보다 많이 듭니다. 처음엔 지역구 의원이어도 후원회를 열지 않아도 되지 않을까? 더 보기</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
+          <t>밤이 오고 기온이 떨어져 집회에 참여한 시민들을 고려해 밤 9시20분 탄핵투표를 종료하였습니다. 과연 나는 최선을 다했나 반성합니다. 오늘 실망을 드려 죄송합니다. 그러나 끝까지 싸워 윤석열ㆍ김건희정권을 끝장내겠습니다.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+          <t>민주당을 171석 제 1당으로 만들어준 국민께서 어처구니 없는 친위 쿠데타를 일단 막으신 겁니다. 깊이 깊이 감사드립니다.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(minhee.official)</t>
+          <t>X(@minhee_choi_)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1334,12 +1334,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>최민희 5시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 1천 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 4시간</t>
+          <t>국회의원도 잘못하면 국민이 소환할 수 있게 ‘국회의원 국민소환법’을 발의했습니다! 22대 국회가 이 법을 통과시키도록 같이 힘모아주세요! "투표 통과하면 의원직 상실"...최민희, 국민소환제 법안 발의 보낸 사람: v.daum.net</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+          <t>https://x.com/minhee_choi_</t>
         </is>
       </c>
     </row>
@@ -1351,20 +1351,74 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>X(@minhee_choi_)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>내란사태가 터졌는데 내란수괴가 멀쩡하고 공범들도 무탈하고 국힘 대표도 건재하고 원내대표도 추경호 그대로다. 이게 무슨 일인가.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://x.com/minhee_choi_</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>확인불가</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>최민희 5시간 [한 표 줍쑈!] 당대표경선투표시작! [당대표] 3번 당원바라기 정청래, [최고위원]언론개혁 10번최민희ㆍ 검찰개혁 3번이성윤ㆍ 당원주권 8번 한민수! 1천 박홍진 고 이해찬 님도 ㅡ한표줍쇼 우리 민희도 ㅡ한표 줍쇼 4시간</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0YYRHrTiKTy4AB4DXhnEe28mMkua2My2AQzoNZ1LQ9Y2xwwu6zdCFHXJcM7mzJcgVl</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>확인불가</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>최민희 2시간 [김민석후보님, 신천지가 민주당 전대에 개입한 근거있다구요?깜놀 입니다. 근거를 즉시 공개하고 신천지개입을 선제차단하십시다! [적절한 시기]에 공개한다니, [지금]이 [적절한 시기]인 거 모르세요? 1천 심화섭 근거가 있음 선제적으로 문제해결을 해야지요. 쥐고 있을 이유는 없습니다. 1시간</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid02fT13wrpb8dM61CCahVNjR7LetrvTm7J1rrohDRfRk4EXhr5Evsm9hyoctwWLcxHil</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 13:57 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,52 +453,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>37m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7월 20일</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 15:49 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>37m</t>
+          <t>12시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
         </is>
       </c>
     </row>
@@ -490,12 +490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>7월 20일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -507,52 +507,106 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>37m</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7월 20일</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 17:25 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,54 +453,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12시간</t>
+          <t>4h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>12시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>37m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -544,12 +544,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7월 20일</t>
+          <t>37m</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -561,52 +561,79 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>7월 20일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-21 21:14 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4h</t>
+          <t>7h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -480,54 +480,54 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>12시간</t>
+          <t>4h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>12시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>37m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7월 20일</t>
+          <t>37m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -588,52 +588,79 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>7월 20일</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 00:04 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>7h</t>
+          <t>18분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 8.17 전대는 심플합니다. 1.검찰개혁 하느냐? 마느냐? 2.1인1표제 사수냐? 파기냐? 3.김대중, 노무현, 문재인, 이재명 대통령의 역사계승의 관점에서 통합이냐? 분열이냐? 분열주의적 음모론을 넘어 통합과 개혁으로 갑시다.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TVQhDwQ6VLXu21ZuaniEbfX6o7CA9jWERaJEAZfiqtr5Ud8kwRdmXAFW9jzVmnrfl</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4h</t>
+          <t>10h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -507,27 +507,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12시간</t>
+          <t>7h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>4h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -561,27 +561,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>37m</t>
+          <t>12시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
         </is>
       </c>
     </row>
@@ -598,12 +598,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7월 20일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -615,52 +615,106 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>37m</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7월 20일</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 04:23 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,54 +453,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>18분</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 8.17 전대는 심플합니다. 1.검찰개혁 하느냐? 마느냐? 2.1인1표제 사수냐? 파기냐? 3.김대중, 노무현, 문재인, 이재명 대통령의 역사계승의 관점에서 통합이냐? 분열이냐? 분열주의적 음모론을 넘어 통합과 개혁으로 갑시다.</t>
+          <t>이재명 대통령, ‘제3자 뇌물죄’가 잘못됐다고 한다.
+“정치적 목적으로 형벌 제도를 운영하다 이런 지경까지 왔다”면서,
+“어떻게든 정리해야 한다”고 주장했다.
+이재명 대통령이 지적한 ‘제3자 공익 기부’, … 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TVQhDwQ6VLXu21ZuaniEbfX6o7CA9jWERaJEAZfiqtr5Ud8kwRdmXAFW9jzVmnrfl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid06qvLmgjJv9a76YNtkBRbUM9zWwz3AXHnWUZqL2weeYof8iXy5XSSf8pCSDwpm8mMl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>&lt;제309차 최고위원회의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/hbd7851/posts/pfbid0ofhqMj8ztvAUr7tHc3pDjnB74nB4Eg3d8nm6972zH35uytBkpQhrXf2pDnYLA3Nhl</t>
         </is>
       </c>
     </row>
@@ -517,7 +520,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7h</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -534,54 +537,54 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4h</t>
+          <t>18분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>정청래의 알콩달콩 8.17 전대는 심플합니다. 1.검찰개혁 하느냐? 마느냐? 2.1인1표제 사수냐? 파기냐? 3.김대중, 노무현, 문재인, 이재명 대통령의 역사계승의 관점에서 통합이냐? 분열이냐? 분열주의적 음모론을 넘어 통합과 개혁으로 갑시다.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TVQhDwQ6VLXu21ZuaniEbfX6o7CA9jWERaJEAZfiqtr5Ud8kwRdmXAFW9jzVmnrfl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>12시간</t>
+          <t>10h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -598,7 +601,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>7h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -625,7 +628,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>37m</t>
+          <t>4h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -642,79 +645,160 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>7월 20일</t>
+          <t>12시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>7월 19일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>37m</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7월 20일</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7월 19일</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>5시간</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 05:20 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,165 +453,167 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>5h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>이재명 대통령, ‘제3자 뇌물죄’가 잘못됐다고 한다.
-“정치적 목적으로 형벌 제도를 운영하다 이런 지경까지 왔다”면서,
-“어떻게든 정리해야 한다”고 주장했다.
-이재명 대통령이 지적한 ‘제3자 공익 기부’, … 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt; 청년의 삶에 영향을 미치는 정책이라면 그 출발 역시 청년의 목소리여야 합니다. 정부 또한 더욱 섬세하고 획기적인 방안을 늘 고민하지만, 청년 여러분께서 매일 마주하는 현실을 모두 담아내기에는 분명 한계가 있습니다. 이제 청년 여러분을 단지 정책의 대상이 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid06qvLmgjJv9a76YNtkBRbUM9zWwz3AXHnWUZqL2weeYof8iXy5XSSf8pCSDwpm8mMl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>5시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;제309차 최고위원회의&gt;… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/hbd7851/posts/pfbid0ofhqMj8ztvAUr7tHc3pDjnB74nB4Eg3d8nm6972zH35uytBkpQhrXf2pDnYLA3Nhl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iY77kEayf1WPZ4B7eQKVWdgLiYfnBmiGnxwrQaFc9pvtV5JvrgubhCyLSfSMacCWl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>18분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>&lt;엄벌에 처해주시고 배후도 철저하게 밝혀주시기 바랍니다.&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02KQgJksBEVZiNTxETD73q8aqNP398HEAYYHP5cE47xgRW4HWRBuBkBbdYdVk8qyD6l</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>18분</t>
+          <t>44분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 8.17 전대는 심플합니다. 1.검찰개혁 하느냐? 마느냐? 2.1인1표제 사수냐? 파기냐? 3.김대중, 노무현, 문재인, 이재명 대통령의 역사계승의 관점에서 통합이냐? 분열이냐? 분열주의적 음모론을 넘어 통합과 개혁으로 갑시다.</t>
+          <t>강남에 ‘매도자 대출’이 등장했다고 한다.
+이재명식 ‘더불어근저당’이다.
+고가 주택 매매의 ‘뉴노멀’이 될 모양이다.
+강남 부자들 욕하더니 하는 짓은 딱 ‘강남 스타일’이다.… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TVQhDwQ6VLXu21ZuaniEbfX6o7CA9jWERaJEAZfiqtr5Ud8kwRdmXAFW9jzVmnrfl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02zV1LidSJ249MWTyjvxcBd1ifqEAbVYFDyvnVPYTa8Ny6RmLNXHacyjB7dhmeRnp5l</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>&lt;제309차 최고위원회의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/hbd7851/posts/pfbid0ofhqMj8ztvAUr7tHc3pDjnB74nB4Eg3d8nm6972zH35uytBkpQhrXf2pDnYLA3Nhl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>&lt;공정과 상식을 파괴한 주범은 바로 이재명 대통령입니다&gt;
+어제 이재명 대통령이 국무회의에서 ‘불법·편법 부동산 불로소득이 공정과 상식 파괴 주범’이라고 발언했습니다. 대통령의 언어는 최소한의 공감능력마저 상실했습니다.
+본인 아파트를 근저당 끼워서 팔아버린 기상천외한 아파트 외상거래야말로 ‘편법’의 전형입니다. 자신이 만든 대출규제를 자신이 우회하는 기만이야말로 공정과 상식의 파괴입니다. … 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid02H3jEiijrKRYiXyd3uJGBoRrguBW4oUy4ro5GCGqFqAodCVxCZZSfDeYCK4Cgq5mSl</t>
         </is>
       </c>
     </row>
@@ -628,7 +630,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4h</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -645,162 +647,54 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12시간</t>
+          <t>57분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 민주, '정청래 암살단 모집' 의혹에 경찰 수사·신변보호 요청. 정청래 “후보 차량 습격 당해 파손…경찰 조사 중”...암살단에 이어서 차량습격. 12.3 비상계엄때는 노상원 수첩에 의해 죽을뻔했는데...참담하고 서글픕니다. 2.8천 1.1천</t>
+          <t>최민희 [호남 역전!] 정청래 25.7% 김민석 21.5% 당원님들, 1인1표의 위엄을 보여주십시오!!!! 오안배 응원합니다</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0aXCYchaZ22685YfQJz68jzXiVBEqFjuzk8BAqyGwET5xfdyPA27GPxzQdHfscAt3l</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02aHYiJ9LZYQqFFCt53u6ftLoBph3cnvaARupkcMbV5TUZfiJBr9etQy5kGHnUMTmWl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>과방위원장(최민희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(minhee.official)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>2분</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+          <t>"김민석 후보, '신천지 개입' 근거를 내놓으세요!"</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>37m</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7월 20일</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>&lt;좋은 질문이 긍정적인 변화를 만듭니다&gt; 오늘은 조금 특별한 하루였습니다. 오전에는 과학기술정보통신부의 젊은 직원들과 타운홀 미팅을 했고, 이어 취임 1주년을 맞아 출입기자단과 기자간담회를 가졌습니다. 하루 종일 질문을 듣고 답을 하면서, 오히려 제가 더 많은 것을 배우는 더 보기</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>대통령(이재명)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>X(@Jaemyung_Lee)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7월 19일</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>백범 김구 선생께서는 부강한 나라보다 높은 문화의 힘으로 인류에 공헌하는 나라를 꿈꾸셨습니다. 인류 불행의 근원을 인간의 내면에서 찾으셨고, 이를 극복할 수 있는 길은 오직 문화에 있다고 역설하셨습니다. "평화의 방벽은 인간의 마음속에 세워야 한다." 유네스코 헌장이 선언한 이 정신은 더 보기 00:34</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://x.com/Jaemyung_Lee</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>5시간</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>&lt;제89차 원내대책회의&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/hbd7851/posts/pfbid0u8XJsfdC6Vr1tRS5458D1SMEQjtDZ392eHz5VBaR6eXC711RehnFpLb2brCbtzGcl</t>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid0UTKoDhphp98aZt6utdnG2egLpMCDCvFr6zBkKW21RgiwmDHvRRHWGcMP9jiVenH1l</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 07:38 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,101 +453,155 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt; 청년의 삶에 영향을 미치는 정책이라면 그 출발 역시 청년의 목소리여야 합니다. 정부 또한 더욱 섬세하고 획기적인 방안을 늘 고민하지만, 청년 여러분께서 매일 마주하는 현실을 모두 담아내기에는 분명 한계가 있습니다. 이제 청년 여러분을 단지 정책의 대상이 더 보기</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 개시</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>5시간</t>
+          <t>22h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 3편 공개</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iY77kEayf1WPZ4B7eQKVWdgLiYfnBmiGnxwrQaFc9pvtV5JvrgubhCyLSfSMacCWl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>18분</t>
+          <t>5h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;엄벌에 처해주시고 배후도 철저하게 밝혀주시기 바랍니다.&gt;… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt; 청년의 삶에 영향을 미치는 정책이라면 그 출발 역시 청년의 목소리여야 합니다. 정부 또한 더욱 섬세하고 획기적인 방안을 늘 고민하지만, 청년 여러분께서 매일 마주하는 현실을 모두 담아내기에는 분명 한계가 있습니다. 이제 청년 여러분을 단지 정책의 대상이 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02KQgJksBEVZiNTxETD73q8aqNP398HEAYYHP5cE47xgRW4HWRBuBkBbdYdVk8qyD6l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>5시간</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iY77kEayf1WPZ4B7eQKVWdgLiYfnBmiGnxwrQaFc9pvtV5JvrgubhCyLSfSMacCWl</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>18분</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>&lt;엄벌에 처해주시고 배후도 철저하게 밝혀주시기 바랍니다.&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02KQgJksBEVZiNTxETD73q8aqNP398HEAYYHP5cE47xgRW4HWRBuBkBbdYdVk8qyD6l</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>44분</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>강남에 ‘매도자 대출’이 등장했다고 한다.
 이재명식 ‘더불어근저당’이다.
@@ -555,144 +609,144 @@
 강남 부자들 욕하더니 하는 짓은 딱 ‘강남 스타일’이다.… 더 보기</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid02zV1LidSJ249MWTyjvxcBd1ifqEAbVYFDyvnVPYTa8Ny6RmLNXHacyjB7dhmeRnp5l</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>3시간</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>&lt;제309차 최고위원회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0ofhqMj8ztvAUr7tHc3pDjnB74nB4Eg3d8nm6972zH35uytBkpQhrXf2pDnYLA3Nhl</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>4시간</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>&lt;공정과 상식을 파괴한 주범은 바로 이재명 대통령입니다&gt;
 어제 이재명 대통령이 국무회의에서 ‘불법·편법 부동산 불로소득이 공정과 상식 파괴 주범’이라고 발언했습니다. 대통령의 언어는 최소한의 공감능력마저 상실했습니다.
 본인 아파트를 근저당 끼워서 팔아버린 기상천외한 아파트 외상거래야말로 ‘편법’의 전형입니다. 자신이 만든 대출규제를 자신이 우회하는 기만이야말로 공정과 상식의 파괴입니다. … 더 보기</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jsjeong0403/posts/pfbid02H3jEiijrKRYiXyd3uJGBoRrguBW4oUy4ro5GCGqFqAodCVxCZZSfDeYCK4Cgq5mSl</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>15h</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>과방위원장(최민희)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Facebook(minhee.official)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>57분</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>최민희 [호남 역전!] 정청래 25.7% 김민석 21.5% 당원님들, 1인1표의 위엄을 보여주십시오!!!! 오안배 응원합니다</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02aHYiJ9LZYQqFFCt53u6ftLoBph3cnvaARupkcMbV5TUZfiJBr9etQy5kGHnUMTmWl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15h</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>과방위원장(최민희)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>57분</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>최민희 [호남 역전!] 정청래 25.7% 김민석 21.5% 당원님들, 1인1표의 위엄을 보여주십시오!!!! 오안배 응원합니다</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02aHYiJ9LZYQqFFCt53u6ftLoBph3cnvaARupkcMbV5TUZfiJBr9etQy5kGHnUMTmWl</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>2분</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>"김민석 후보, '신천지 개입' 근거를 내놓으세요!"</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0UTKoDhphp98aZt6utdnG2egLpMCDCvFr6zBkKW21RgiwmDHvRRHWGcMP9jiVenH1l</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 08:51 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,155 +453,209 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>15분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 개시</t>
+          <t>&lt;모처럼 방송촐연했습니다.&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid035Dn9rYMFo8hUVzPpaSZWcS9Xhz4D2X1hMzqyWsbhrTPnMjFzwrRC94APbBhSiJxtl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22h</t>
+          <t>41분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 3편 공개</t>
+          <t>&lt;검찰개혁은 시대적 요구입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/reel/1675336690239600/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt; 청년의 삶에 영향을 미치는 정책이라면 그 출발 역시 청년의 목소리여야 합니다. 정부 또한 더욱 섬세하고 획기적인 방안을 늘 고민하지만, 청년 여러분께서 매일 마주하는 현실을 모두 담아내기에는 분명 한계가 있습니다. 이제 청년 여러분을 단지 정책의 대상이 더 보기</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 개시</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5시간</t>
+          <t>22h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 3편 공개</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iY77kEayf1WPZ4B7eQKVWdgLiYfnBmiGnxwrQaFc9pvtV5JvrgubhCyLSfSMacCWl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18분</t>
+          <t>5h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;엄벌에 처해주시고 배후도 철저하게 밝혀주시기 바랍니다.&gt;… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt; 청년의 삶에 영향을 미치는 정책이라면 그 출발 역시 청년의 목소리여야 합니다. 정부 또한 더욱 섬세하고 획기적인 방안을 늘 고민하지만, 청년 여러분께서 매일 마주하는 현실을 모두 담아내기에는 분명 한계가 있습니다. 이제 청년 여러분을 단지 정책의 대상이 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02KQgJksBEVZiNTxETD73q8aqNP398HEAYYHP5cE47xgRW4HWRBuBkBbdYdVk8qyD6l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>5시간</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iY77kEayf1WPZ4B7eQKVWdgLiYfnBmiGnxwrQaFc9pvtV5JvrgubhCyLSfSMacCWl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>18분</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>&lt;엄벌에 처해주시고 배후도 철저하게 밝혀주시기 바랍니다.&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02KQgJksBEVZiNTxETD73q8aqNP398HEAYYHP5cE47xgRW4HWRBuBkBbdYdVk8qyD6l</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>44분</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>강남에 ‘매도자 대출’이 등장했다고 한다.
 이재명식 ‘더불어근저당’이다.
@@ -609,144 +663,144 @@
 강남 부자들 욕하더니 하는 짓은 딱 ‘강남 스타일’이다.… 더 보기</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid02zV1LidSJ249MWTyjvxcBd1ifqEAbVYFDyvnVPYTa8Ny6RmLNXHacyjB7dhmeRnp5l</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Facebook(hbd7851)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>3시간</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>&lt;제309차 최고위원회의&gt;… 더 보기</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/hbd7851/posts/pfbid0ofhqMj8ztvAUr7tHc3pDjnB74nB4Eg3d8nm6972zH35uytBkpQhrXf2pDnYLA3Nhl</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>4시간</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>&lt;공정과 상식을 파괴한 주범은 바로 이재명 대통령입니다&gt;
 어제 이재명 대통령이 국무회의에서 ‘불법·편법 부동산 불로소득이 공정과 상식 파괴 주범’이라고 발언했습니다. 대통령의 언어는 최소한의 공감능력마저 상실했습니다.
 본인 아파트를 근저당 끼워서 팔아버린 기상천외한 아파트 외상거래야말로 ‘편법’의 전형입니다. 자신이 만든 대출규제를 자신이 우회하는 기만이야말로 공정과 상식의 파괴입니다. … 더 보기</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jsjeong0403/posts/pfbid02H3jEiijrKRYiXyd3uJGBoRrguBW4oUy4ro5GCGqFqAodCVxCZZSfDeYCK4Cgq5mSl</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>15h</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>과방위원장(최민희)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook(minhee.official)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>57분</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>최민희 [호남 역전!] 정청래 25.7% 김민석 21.5% 당원님들, 1인1표의 위엄을 보여주십시오!!!! 오안배 응원합니다</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/minhee.official/posts/pfbid02aHYiJ9LZYQqFFCt53u6ftLoBph3cnvaARupkcMbV5TUZfiJBr9etQy5kGHnUMTmWl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>X(@msitminister)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>15h</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>&lt;국제생물·화학올림피아드 전원 메달, 진심으로 축하합니다&gt; 대한민국 과학인재들이 또 한 번 세계 무대에서 대한민국 과학의 저력을 보여주었습니다. 국제생물올림피아드에서는 대표학생 4명 전원이 금메달을, 국제화학올림피아드에서는 대표학생 4명 모두가 금메달 2개, 은메달 1개, 동메달 1개를 더 보기</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://x.com/msitminister</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>과방위원장(최민희)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Facebook(minhee.official)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>57분</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>최민희 [호남 역전!] 정청래 25.7% 김민석 21.5% 당원님들, 1인1표의 위엄을 보여주십시오!!!! 오안배 응원합니다</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/minhee.official/posts/pfbid02aHYiJ9LZYQqFFCt53u6ftLoBph3cnvaARupkcMbV5TUZfiJBr9etQy5kGHnUMTmWl</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>과방위원장(최민희)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Facebook(minhee.official)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>2분</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>"김민석 후보, '신천지 개입' 근거를 내놓으세요!"</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>https://www.facebook.com/minhee.official/posts/pfbid0UTKoDhphp98aZt6utdnG2egLpMCDCvFr6zBkKW21RgiwmDHvRRHWGcMP9jiVenH1l</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 12:30 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,79 +453,133 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-22 15:10 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -458,103 +458,103 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -566,20 +566,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-23 02:54 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -485,103 +485,103 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -593,20 +593,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-23 05:58 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,187 +453,241 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-23 14:06 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,204 +490,258 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-23 16:36 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,54 +453,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -512,22 +512,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -539,209 +539,290 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-23 20:17 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -485,49 +485,49 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -539,22 +539,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -566,12 +566,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -593,22 +593,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -620,12 +620,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -635,61 +635,61 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -701,103 +701,103 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -809,20 +809,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 04:18 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -458,61 +458,61 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -522,66 +522,66 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -598,17 +598,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -625,12 +625,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -652,204 +652,258 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 07:36 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -485,22 +485,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -517,44 +517,44 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -566,49 +566,49 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -620,22 +620,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -674,22 +674,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -701,12 +701,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -716,61 +716,61 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -782,103 +782,103 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -890,20 +890,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 10:22 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,81 +453,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -539,61 +539,61 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -603,66 +603,66 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -679,17 +679,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -733,204 +733,258 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 12:24 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,297 +453,299 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>23h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
+재판도 생방송으로 공개하는 세상이다.
+선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -755,22 +757,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -782,209 +784,290 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 15:01 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -458,117 +458,117 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -578,93 +578,93 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -676,61 +676,61 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -740,66 +740,66 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -816,17 +816,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -843,12 +843,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -870,204 +870,258 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 18:23 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -458,159 +458,159 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -622,76 +622,76 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -703,22 +703,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -735,44 +735,44 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -784,49 +784,49 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -838,22 +838,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -892,22 +892,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -919,12 +919,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -934,61 +934,61 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1000,103 +1000,103 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1108,20 +1108,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-24 22:08 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -485,159 +485,159 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -649,76 +649,76 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -730,22 +730,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -762,44 +762,44 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -811,49 +811,49 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -865,22 +865,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -892,12 +892,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -919,22 +919,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -961,61 +961,61 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1027,103 +1027,103 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1135,20 +1135,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-25 04:15 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -485,76 +485,76 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -588,353 +588,353 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -946,22 +946,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -973,209 +973,290 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-25 07:22 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,71 +490,71 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -566,76 +566,76 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -669,353 +669,353 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1054,209 +1054,290 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-25 09:51 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,81 +453,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -539,184 +539,184 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -728,117 +728,117 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -848,93 +848,93 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -946,61 +946,61 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1010,66 +1010,66 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1086,17 +1086,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1140,204 +1140,258 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-25 13:39 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,12 +453,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,12 +468,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -485,12 +485,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -500,34 +500,34 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -539,76 +539,76 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -620,103 +620,103 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -728,159 +728,159 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -892,76 +892,76 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -973,22 +973,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1005,44 +1005,44 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1054,49 +1054,49 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1108,22 +1108,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1135,12 +1135,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1162,22 +1162,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1189,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1204,61 +1204,61 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1270,103 +1270,103 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1378,20 +1378,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-26 02:57 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,162 +453,162 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -620,184 +620,184 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -809,117 +809,117 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -929,93 +929,93 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1027,61 +1027,61 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1091,66 +1091,66 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1221,204 +1221,258 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-26 06:10 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,216 +453,216 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -674,184 +674,184 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -863,117 +863,117 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -983,93 +983,93 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1081,61 +1081,61 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1145,66 +1145,66 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1248,12 +1248,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1275,204 +1275,258 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-26 13:28 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,147 +453,147 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -603,12 +603,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -620,12 +620,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -635,34 +635,34 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -674,76 +674,76 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -755,103 +755,103 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -863,159 +863,159 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1027,76 +1027,76 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1108,22 +1108,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1140,44 +1140,44 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1189,49 +1189,49 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1243,22 +1243,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1270,12 +1270,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1297,22 +1297,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1324,12 +1324,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1339,61 +1339,61 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1405,103 +1405,103 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1513,20 +1513,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-27 04:40 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,174 +453,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -630,12 +630,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -662,34 +662,34 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -701,76 +701,76 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -782,103 +782,103 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -890,159 +890,159 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1054,76 +1054,76 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1167,44 +1167,44 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1216,49 +1216,49 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1270,22 +1270,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1297,12 +1297,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1324,22 +1324,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1351,12 +1351,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1366,61 +1366,61 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1432,103 +1432,103 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1540,20 +1540,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-27 08:34 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -480,297 +480,297 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -782,184 +782,184 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -971,117 +971,117 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1091,93 +1091,93 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1189,61 +1189,61 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1253,66 +1253,66 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1329,17 +1329,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1356,12 +1356,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1383,204 +1383,258 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-27 12:31 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,201 +453,201 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -657,12 +657,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -696,147 +696,147 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,93 +846,93 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -944,76 +944,76 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1025,495 +1025,495 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Facebook(jkim386.kmcc)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>13시간</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2h</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>방통위(김종철)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>X(@jkim386_kmcc)</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>6m</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>https://x.com/jkim386_kmcc</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>방통위(김종철)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Facebook(jkim386.kmcc)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2시간</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1523,24 +1523,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1567,49 +1567,49 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1626,15 +1626,177 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>15시간</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>14시간</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Facebook(jkim386.kmcc)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 02:40 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,135 +453,135 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
@@ -593,277 +593,277 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -890,12 +890,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -905,34 +905,34 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -944,76 +944,76 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1025,103 +1025,103 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1133,159 +1133,159 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1297,76 +1297,76 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1378,22 +1378,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1410,44 +1410,44 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1459,49 +1459,49 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1540,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1567,22 +1567,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1594,12 +1594,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1609,61 +1609,61 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1675,103 +1675,103 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1783,20 +1783,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 05:50 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,162 +453,162 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
@@ -620,277 +620,277 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -917,12 +917,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -932,34 +932,34 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -971,76 +971,76 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1052,103 +1052,103 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1160,159 +1160,159 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1324,76 +1324,76 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1405,22 +1405,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1437,44 +1437,44 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1486,49 +1486,49 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1540,22 +1540,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1594,22 +1594,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1636,61 +1636,61 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1702,103 +1702,103 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1810,20 +1810,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 14:14 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,162 +453,162 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -620,319 +620,319 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
@@ -949,71 +949,71 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1047,12 +1047,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,24 +1062,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1089,93 +1089,93 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1187,591 +1187,591 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>13시간</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>X(@msitminister)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2h</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://x.com/msitminister</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>방통위(김종철)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>X(@jkim386_kmcc)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>6m</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1788,17 +1788,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1810,47 +1810,182 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>14시간</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 16:46 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>14m</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,12 +490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>13h</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -507,54 +507,54 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
@@ -566,211 +566,211 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
@@ -782,277 +782,277 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1094,34 +1094,34 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1133,76 +1133,76 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1214,103 +1214,103 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1322,159 +1322,159 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1486,76 +1486,76 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1567,22 +1567,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1599,44 +1599,44 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1648,49 +1648,49 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1702,22 +1702,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1756,22 +1756,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1798,61 +1798,61 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1864,103 +1864,103 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1972,20 +1972,47 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 18:19 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>53m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
+          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,12 +490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>14m</t>
+          <t>17h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -507,135 +507,135 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>13h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
+          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
@@ -647,346 +647,346 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1003,206 +1003,206 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1219,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1246,71 +1246,71 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1322,76 +1322,76 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1425,353 +1425,353 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1783,22 +1783,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1810,209 +1810,290 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 20:20 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>53m</t>
+          <t>19h</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,12 +490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>53m</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
+          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -507,54 +507,54 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>17h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
+          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14m</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>13h</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -615,54 +615,54 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
@@ -674,211 +674,211 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
@@ -890,277 +890,277 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1170,12 +1170,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1202,34 +1202,34 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1241,76 +1241,76 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1322,103 +1322,103 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1430,159 +1430,159 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>37분</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
@@ -1594,76 +1594,76 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1675,22 +1675,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
@@ -1707,44 +1707,44 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
@@ -1756,49 +1756,49 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1810,22 +1810,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1837,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
@@ -1864,22 +1864,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1891,12 +1891,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1906,61 +1906,61 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
@@ -1972,103 +1972,103 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -2080,20 +2080,47 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-28 22:09 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19h</t>
+          <t>7m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
+          <t>룰라 브라질 대통령이 노동조합 위원장으로 일하던 노조사무실에 방문했습니다. 노동이 존중되는 세상을 만드는 일은 브라질이나 대한민국이나 다를 것이 없습니다.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,12 +490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>53m</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
+          <t>지구 반대편 땅에서 개척의 역사를 써 내려가신 자랑스러운 브라질 재외동포 여러분께 인사드렸습니다. 아리랑 농장의 푸른 들판에서부터 상파울루의 섬유, 패션 산업에 이르기까지 우리 동포 여러분의 뜨거운 열정이 브라질 곳곳에 남아 있습니다. 낯선 땅에서도 성실함과 끈기로 새 길을 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -517,12 +517,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>21h</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 7월 27일 Hoje tive a honra de receber o presi</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -534,27 +534,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>19h</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>53m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
+          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14m</t>
+          <t>17h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -615,135 +615,135 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
+          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
@@ -755,346 +755,346 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1111,206 +1111,206 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1354,71 +1354,71 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1430,76 +1430,76 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1533,353 +1533,353 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1891,22 +1891,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1918,209 +1918,290 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-29 00:03 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>7m</t>
+          <t>55m</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>룰라 브라질 대통령이 노동조합 위원장으로 일하던 노조사무실에 방문했습니다. 노동이 존중되는 세상을 만드는 일은 브라질이나 대한민국이나 다를 것이 없습니다.</t>
+          <t>남미 경제의 심장, 브라질 상파울루에서 양국의 미래를 함께 만들어 갈 기업인 여러분을 만났습니다. 브라질은 대한민국의 남미 최대 교역국이자 우리 기업들이 활발히 진출해 있는 나라입니다. 대한민국의 뛰어난 기술과 제조 역량이 브라질의 풍부한 자원, 성장 잠재력과 만난다면 양국은 더 보기</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -485,49 +485,49 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>21시간</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>지구 반대편 땅에서 개척의 역사를 써 내려가신 자랑스러운 브라질 재외동포 여러분께 인사드렸습니다. 아리랑 농장의 푸른 들판에서부터 상파울루의 섬유, 패션 산업에 이르기까지 우리 동포 여러분의 뜨거운 열정이 브라질 곳곳에 남아 있습니다. 낯선 땅에서도 성실함과 끈기로 새 길을 더 보기</t>
+          <t>&lt;지구 반대편 브라질에서 대한민국 경제와 외교의 지평을 넓혀갑니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0CghEaiKD7bqfFgtRKuafzV8ScTiNNhYBbDEc281Z7pRb1xEfECLeeh3AnnqJUrVXl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 7월 27일 Hoje tive a honra de receber o presi</t>
+          <t>&lt;여론은 추세가 중요하다.&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid07qhNdFP6REWoTDM4dWXDDZa6e1er381fqU64RAoyce5bWug13LwRKWLgRrHpwMSkl</t>
         </is>
       </c>
     </row>
@@ -544,12 +544,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>19h</t>
+          <t>7m</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
+          <t>룰라 브라질 대통령이 노동조합 위원장으로 일하던 노조사무실에 방문했습니다. 노동이 존중되는 세상을 만드는 일은 브라질이나 대한민국이나 다를 것이 없습니다.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>53m</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
+          <t>지구 반대편 땅에서 개척의 역사를 써 내려가신 자랑스러운 브라질 재외동포 여러분께 인사드렸습니다. 아리랑 농장의 푸른 들판에서부터 상파울루의 섬유, 패션 산업에 이르기까지 우리 동포 여러분의 뜨거운 열정이 브라질 곳곳에 남아 있습니다. 낯선 땅에서도 성실함과 끈기로 새 길을 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>21h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 7월 27일 Hoje tive a honra de receber o presi</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -615,27 +615,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>19h</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>53m</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
+          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14m</t>
+          <t>17h</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -696,135 +696,135 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13h</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
+          <t>&lt;전북 지체장애인 협회 간담회&gt;</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid02N14ho4CoR1gScDZU4eoLowEjuQPZu8D2GSZwJoeUCgjnNAcpM9SGJdxGSmsazRUrl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>7시간</t>
+          <t>15h</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 19h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
+          <t>"만나서 반갑습니다"보다 "그동안 잘 지내셨습니까"가 더 자연스러운 사이가 되었습니다. 오랜 친구를 맞이하듯 반갑게 맞아주신 @LulaOficial 대통령님께 특별한 감사를 전합니다. 만남이 거듭될수록 서로를 향한 믿음은 깊어지고, 함께 그려갈 미래 역시 선명해지고 있습니다. 그동안 우리가 더 보기 [4K HDR] 감사합니다, 브라질!🇰🇷🇧🇷 | 브라질 국빈 방문 보낸 사람: youtube.com</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>13h</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
+          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 16h Hoje tive a honra de receber o presiden</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>7시간</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>도대체 국회의장까지 왜 이러실까요?… 더 보기</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jsjeong0403/posts/pfbid023Yb1YWHuY79qwKMBcKTyP6Sb2nkKYiPyjoGrLxw4Fbzsoobp5ZMsAFWfAnnVS2oml</t>
         </is>
       </c>
     </row>
@@ -836,346 +836,346 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt; 일부 커피 프랜차이즈 업체가 시스템 업그레이드나 앱 개편을 이유로 소비자들이 쌓아 올린 소중한 구매적립 이력을 명확한 고지 없이 일방적으로 소멸시킨 사례가 발생하였습니다. 이러한 생활 밀착형 플랫폼 서비스의 맹점과 이용자 피해에 대해 더 보기</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02pcK6CxN4CoKZL91yRh6CkGRaed93n7sKVfjV9JqSXodNzdfrheQ1NKdgDK21HF1al</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
+          <t>EU 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0LsKapGkdy1qxNPZUaPwjYvN8WFAn6gwM4mYWcEHg1LQzRpTPKTAa1neQBKCTwPdvl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>더불어민주당 원내대표(한병도)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Facebook(hbd7851)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>21분</t>
+          <t>17시간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
+          <t>신규 휴대폰 사전예약 관련 허위·과장 광고에 대한 소비자 주의 당부</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/2835946096774008/</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0MGumW3mxVqjesoiaKUG99MRFSyQc87vYU4u3kq26Uf6hDbkLu7YrGRNSencJnfEkl</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>국민의힘 원내대표(정점식)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Facebook(jsjeong0403)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
+          <t>프랑스와 스페인에서 계속되고 있는 산불로 큰 피해가 발생하고 있다는 소식에 안타까움을 금할 수 없습니다. 예기치 못한 재난으로 어려움을 겪고 계신 모든 분들께 위로의 말씀을 전합니다. 아울러 위험을 무릅쓰고 산불 진화와 구조 활동에 헌신하고 계신 구조대원과 관계자 여러분께 경의를 더 보기</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/reel/1413933267450382/</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
+          <t>&lt;7월 28일(화) 일정 입니다.&gt;</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0TV5s7ycUagqxBAu7HesoykaQn3M4dxNzCVj7pYAAzDJ2bGtQWpsKY3JBwSgrTgHul</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>21분</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
+          <t>&lt;민주당의 기준은 오직 국민이고, 민생입니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
+          <t>https://www.facebook.com/reel/2835946096774008/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>국민의힘 원내대표(정점식)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jsjeong0403)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
+          <t>&lt;국민의힘 최고위원회의(7.27)&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/1413933267450382/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02RJWUyryXAhFQp2fm6MwGN7FEmN32PMYRroR7TZCV6cgxJFwU8xWxUkFUuy9LrHSfl</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>국민의힘 대표(장동혁)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Facebook(dhjang6971)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10시간</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
+          <t>샌프란시스코 AI 서밋 참석 및 AI 혁신도시 방문을 통한 도시 혁신 방안 모색</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
+          <t>유럽연합(EU) 집행위원회의 한국에 대한 GDPR 적정성 결정 유지 발표</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02QtvJJ5xCe8itzM23rWnZUUFeXAYNzXW6qGp8HSV55sLckXkALmgjk5GUX6JcRpsQl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>22시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
+          <t>국내 통신 3사와의 AI 네트워크 전략 논의 및 미국 AMD와의 AI 반도체 생태계 협력 MOU 체결</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
@@ -1192,206 +1192,206 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>12분</t>
+          <t>10시간</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
+          <t>전자투표 도입 추진에 대한 비판 및 선거 전산 시스템의 신뢰성 의혹 제기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid0QdJa2KvbK8eT1YWcLX72gWB2Z49jQdXiwJSyCk8LtJKiLyiSQgvoMq11Q4mUJgPDl</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026년 디지털윤리주간 운영 계획</t>
+          <t>샌프란시스코에서 선포한 대한민국의 새로운 AI 시대 비전</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vJnKjkAwN7iBVDnnumCMM2zrgcj5q9C2DWpJ9L62NBK5iTZzvYpjX1ec2CG5gfbbl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>22시간</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
+          <t>유럽연합(EU)의 대한민국 GDPR 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0M3Ub7R2NnevkkE5CAotGCf3eYYfAwi7hoFdScEiPmzAhXT5ih1T1Pmy3MSCeik7Al&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(dhjang6971)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>12분</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>전자투표 도입 정책 및 선거 관리 전산 시스템의 신뢰성 문제</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/dhjang6971/posts/pfbid02UeuHW989z8XRfxDCN5XeV6UKx19RF57MixAV9FeRi13ERHWSJgQwNWtJKjaA3WHKl</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>2일</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
+          <t>2026년 디지털윤리주간 운영 계획</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bP15nXaPPm62VrdJmWGugxhj6SdzEA2CaAHJs3ZFVDmMkAT8fYmVZRp9un5ewQiXl</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
+          <t>샌프란시스코 AI 서밋 참석 및 글로벌 AI 기업 CEO들과의 만찬 회동</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>4시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>54m</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
+          <t>EU 집행위원회의 한국 대상 GDPR(일반개인정보보호법) 적정성 결정 유지</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02Qb7n2aejdputRQRn1ARBC5cJF23PLLptxAYjyRigAuihCmrVuVz31Lqph7DjYScwl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1408,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
+          <t>인간과 AI의 조화로운 공존 및 미래 성장을 위한 국제사회 협력 제안</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1435,71 +1435,71 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>4시간</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
+          <t>샌프란시스코에서의 대한민국 새로운 AI 시대 비전 선포 및 글로벌 협력</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02yrRWeuoJDQfJ87yRvCrBmYCZy1xtAL2X2iE2eCrG1TDFewmBUfe74eab3dphscA1l</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>54m</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 계획</t>
+          <t>국내외 주요 테크 기업들이 참여하여 협력 의제를 발굴하는 '샌프란시스코 AI 서밋' 개최</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>13시간</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
+          <t>글로벌 AI 기업 대표들과의 협력 및 AI 시대의 미래 논의</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
@@ -1511,76 +1511,76 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
+          <t>대한민국의 새로운 글로벌 AI 시대 비전 선포</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0vUwL2tSgBcBAb13EafDhoCvXTYr6GeCg8gpUTskf94pYVsEUaSZqK9gAu6xFbBVkl</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2일</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 계획</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02eveGhhCkF34oCQSNc56ovrCLA4NscQc318gcfCheGn45oDtBBRK1EJQSagAyPujil</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>37분</t>
+          <t>13시간</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+          <t>개인정보 보호 관념과 미래사회의 새로운 권리를 논의하는 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02UEz5EXCQqDMDE5sRuvugiTJQNuQ6Ze9ia7Xq84jUQwG2FuCWgUNTvzypnEhXX4Uzl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1597,12 +1597,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+          <t>이번 정류장은 샌프란시스코입니다 🇰🇷🇺🇸 youtube.com/shorts/u4Yg1dk… #이재명 #대통령 #US #sanfrancisco #california 00:45</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1614,353 +1614,353 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Facebook(jaemyunglee)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2일</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0epJvXvgszRU3ovjesXbYBv6uFb5mQDCKg8ez8bRq77E2SqSgHPFNSgTArv1nVBzhl</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>37분</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>정청래의 알콩달콩 與, '보완수사권 폐지' 형소법 개정안 당론 추인, 30일 처리할듯…검사는 수사하지 않는다. 검사는 기소만한다. 경찰이 수사한다. 수사기소분리의 대원칙을 당론으로 채택했으니 곧 국회통과. 검찰개혁, 역사의 문턱을 넘습니다. 설악산 고생하셨습니다</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0FHwuim9N2Yqpb5iLZYxTHS31xrwHPW1tdvx28jRoFzeWeohzekwHdcgAkKUDAA6kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>대통령(이재명)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>X(@Jaemyung_Lee)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 7월 23일 ㅋㅋ 00:42</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://x.com/Jaemyung_Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>국민의힘 대표(장동혁)</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Facebook(dhjang6971)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>2시간</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>중앙선관위에서 선거소청 방송 중계를 끝내 거부했다.
 재판도 생방송으로 공개하는 세상이다.
 선거소청을 공개하지 못할 이유가 없다.… 더 보기</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dhjang6971/posts/pfbid0kXyr7RpRSwDJWuFun42koS2zaxwQ7ZfPmNCSvPRe57MZGSXd41EpczMYptxStxL9l</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>더불어민주당 원내대표(한병도)</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Facebook(hbd7851)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/918644363869452/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>X(@kh_song8)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>https://x.com/kh_song8</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>개인정보보호위원회(송경희)</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1시간</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
+          <t>더불어민주당 원내대표(한병도)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>X(@msitminister)</t>
+          <t>Facebook(hbd7851)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
+          <t>&lt;공정한 경쟁, 하나되는 전당대회&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://x.com/msitminister</t>
+          <t>https://www.facebook.com/reel/918644363869452/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>6m</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
+          <t>디지털 시대의 개인정보 권리와 DID 기반 디지털 신원증명 등을 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>'2026년 디지털윤리주간' 운영 소식</t>
+          <t>미래사회의 개인정보 보호와 새로운 권리를 논의하기 위한 '제3차 2026 개인정보 미래포럼' 개최</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0QPYN3rGaywahWzNLaJXiAwWAqVNEAZP7U6WZSygZt2hRpmgMbH5N28xmqWeANFFpl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2h</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>AI 시대 국가 통신 인프라 전략 논의를 위한 통신 3사 CEO 간담회 개최</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3h</t>
+          <t>6m</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
+          <t>안전한 인공지능(AI) 활용 문화 확산 및 디지털 윤리 실천을 위한 '2026년 디지털윤리주간' 운영</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>2시간</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>'2026년 디지털윤리주간' 운영 소식</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0bZA65fr8DL4ZGpecZ58zVqVTA7GvfDEsYLKKF1aMrFHjeNWWf6rxrJ5wzHXkinjFl</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>3시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0oyWP4U5ZjtEusf5CR79pp2evAaiUbMUvjFoPR7ERniXswc43nJSMsvBEkDPF5bkFl</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>3h</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>미안합니다. 김영훈 노동부 장관님. 그런데 장관님이 잠 좀 못 주무시는만큼 누군가 죽을 사람들이 살아남습니다. 열심히 일해 주셔서 진심으로 감사합니다. 장관님 때문에 목숨을 건지고 가정을 지킨 사람들이 참 많습니다. 이경하 @igyeong51134506 5h ㅋㅋ 00:42</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>1일</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid02iMx7T6KEqVSRV1f9xTHmkMJr5yeW9oprvPL3Hf4qFT5dmNhESLJRfLFZkY3Drh9Nl</t>
         </is>
       </c>
     </row>
@@ -1972,22 +1972,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>X(@kh_song8)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>31m</t>
+          <t>3시간</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>오늘 개인정보보호위원회는 공공부문이 AX를 추진하는 과정에서 발생할 수 있는 개인정보 이슈와 필요한 안전조치 등을 담은 「공공 AX 프라이버시 보호 안내서」를 발간했습니다.… 더 보기</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://x.com/kh_song8</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eCGcmoz9nYKUgzs63iMhfqLafKG1NTDxJrJgijux1eg66qR22coTEES1TMP1mb8Sl&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
@@ -1999,209 +1999,290 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>31분</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Facebook(jkim386.kmcc)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15시간</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>방송통신위원회 제24차 전체회의 개최</t>
+          <t>공공부문 AI 전환(AX) 과정의 개인정보 보호 및 안전조치 가이드라인 발간</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02iDsLFdBiTfWvbMKaCdAnDyqnCKxyU1rYbGuT7ru2ZiA3ktxbrrMYVBDcV59thYj4l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>14시간</t>
+          <t>31m</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(profile.php?id=100052519089631)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1h</t>
+          <t>31분</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
+          <t>개인정보보호위원회의 틱톡·애플 대상 개인정보 무단 수집 및 국외 이전에 따른 과징금 부과 및 시정명령 의결</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid0eHqdruqZHzTwNgPDAs6g2bu2Up2XZSBbBue2J26hXijftLSCjvCfmNAncMhC8x36l&amp;id=100052519089631</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+          <t>방송통신위원회 제24차 전체회의 개최</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid02sX9Zydhvb6KWURv2JtWcuSi4j4j5aBkt6BdLDQE4E4rj432GqR7kh1oJ7p3Xbvdcl</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>개인정보보호위원회(송경희)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Facebook(profile.php?id=100052519089631)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1일</t>
+          <t>14시간</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+          <t>&lt;청와대 청년 펠로우를 모십니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0ezTvq4xcowQeVbFF4aBHrTep9pUY5GQ9FxrzwRKB3ypbaMyY1d4vtjRWec8JCuxUl</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>방통위(김종철)</t>
+          <t>대통령(이재명)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>X(@jkim386_kmcc)</t>
+          <t>X(@Jaemyung_Lee)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23h</t>
+          <t>1h</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+          <t>엘살바도르, 콜롬비아, 라오스, 카자흐스탄, 탄자니아, 쿠웨이트, 나이지리아, 브라질의 신임 주한대사들로부터 신임장을 제정받았습니다. 양국 관계가 한층 더 발전할 수 있도록 든든한 가교 역할을 해주시길 부탁드렸습니다. 대한민국에 대한 깊은 애정을 전하며 최선을 다하겠다는 의지를 밝혀주신 더 보기</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://x.com/jkim386_kmcc</t>
+          <t>https://x.com/Jaemyung_Lee</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>더불어민주당 대표(정청래)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Facebook(cheongrae1)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>&lt;잠시후 9시, 2분뉴스 생방송에 출연합니다.&gt;</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cheongrae1/posts/pfbid0HB3iGkr1nmMcTpPN7ThH3uu6dv9WfB2sQCrV1S8R9nn11yzLFmC6PrauXC4UCKzZl</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회(송경희)</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Facebook(profile.php?id=100052519089631)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1일</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>가명정보의 안전한 활용을 지원하는 '개인정보 이노베이션 존' 신규 운영기관 공모 진행</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/permalink.php?story_fbid=pfbid02NeC8U5hNLvAWFJUPDoBbqQFpU9kCDCe5jPCdFbxyAiVPxtgpCcrxzkTXk2wUuyH8l&amp;id=100052519089631</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>방통위(김종철)</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>X(@jkim386_kmcc)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>23h</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>AI 기술을 활용해 불법·허위조작정보 유통 방지 등 방송통신 정책을 소개하는 숏폼 콘텐츠 공개</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://x.com/jkim386_kmcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>방통위(김종철)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>AI 기술을 활용한 방송통신 정책 홍보 숏폼 콘텐츠 '정책플리' 공개</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0ukfx1z5hDzEQ5eanJp4BBgZaPxjeXPPWgxTbxGVsGkXqgXpufSwys3tLa3D2BPpLl</t>
         </is>

</xml_diff>

<commit_message>
auto: SNS 모니터링 업데이트 (2026-07-29 03:33 UTC)
</commit_message>
<xml_diff>
--- a/data/sns_monitoring.xlsx
+++ b/data/sns_monitoring.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -453,162 +453,162 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>과기정통부 장관 겸 과학기술부총리(배경훈)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@msitminister)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>55m</t>
+          <t>7월 27일</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>남미 경제의 심장, 브라질 상파울루에서 양국의 미래를 함께 만들어 갈 기업인 여러분을 만났습니다. 브라질은 대한민국의 남미 최대 교역국이자 우리 기업들이 활발히 진출해 있는 나라입니다. 대한민국의 뛰어난 기술과 제조 역량이 브라질의 풍부한 자원, 성장 잠재력과 만난다면 양국은 더 보기</t>
+          <t>샌프란시스코 AI 서밋 참관 및 AI 기반 도시 혁신 동향</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/msitminister</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>개인정보보호위원회(송경희)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facebook(jaemyunglee)</t>
+          <t>X(@kh_song8)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>21시간</t>
+          <t>7월 25일</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;지구 반대편 브라질에서 대한민국 경제와 외교의 지평을 넓혀갑니다&gt;… 더 보기</t>
+          <t>유럽연합(EU) 집행위원회가 우리나라에 대한 GDPR(유럽연합 일반개인정보보호법) 적정성 결정을 계속 유지하기로 했다고 발표했습니다. 이번 재검토는 2021년 12월 우리나라가 적정성 결정을 받은 이후 처음 실시된 것으로, 쉽게 말하면 우리나라의 개인정보 보호 수준이 유럽연합과 동등한 더 보기</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0CghEaiKD7bqfFgtRKuafzV8ScTiNNhYBbDEc281Z7pRb1xEfECLeeh3AnnqJUrVXl</t>
+          <t>https://x.com/kh_song8</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더불어민주당 대표(정청래)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facebook(cheongrae1)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1시간</t>
+          <t>7월 27일</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;여론은 추세가 중요하다.&gt;… 더 보기</t>
+          <t>&lt;신규 휴대폰 사전예약 과장광고 주의&gt; 8월 7일 삼성전자 '갤럭시Z8 시리즈' 출시에 앞서 내일부터 일주일간 사전 예약이 진행됨에 따라 일부 휴대폰 대리점 및 판매점 등 유통점들의 과도한 지원금과 경품 제공 등에 대한 과장광고가 증가하고 있어 각별한 주의를 부탁드립니다. 사전 예약 기간 및 더 보기</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/cheongrae1/posts/pfbid07qhNdFP6REWoTDM4dWXDDZa6e1er381fqU64RAoyce5bWug13LwRKWLgRrHpwMSkl</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7m</t>
+          <t>7월 24일</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>룰라 브라질 대통령이 노동조합 위원장으로 일하던 노조사무실에 방문했습니다. 노동이 존중되는 세상을 만드는 일은 브라질이나 대한민국이나 다를 것이 없습니다.</t>
+          <t>&lt;'2026년 디지털윤리주간' 운영&gt; 일상 속 인공지능 윤리를 경험하고 실천해 볼 수 있는 다양한 온·오프라인 행사가 전국 각지에서 열리고 있습니다. 방미통위는 안전하고 책임있는 인공지능 활용 문화 확산과 디지털윤리 실천을 위해 '2026년 디지털윤리주간'을 7월 26일(일)까지 운영합니다. 더 보기</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>X(@jkim386_kmcc)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>7월 23일</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>지구 반대편 땅에서 개척의 역사를 써 내려가신 자랑스러운 브라질 재외동포 여러분께 인사드렸습니다. 아리랑 농장의 푸른 들판에서부터 상파울루의 섬유, 패션 산업에 이르기까지 우리 동포 여러분의 뜨거운 열정이 브라질 곳곳에 남아 있습니다. 낯선 땅에서도 성실함과 끈기로 새 길을 더 보기</t>
+          <t>&lt;방미통위 제24차 전체회의 개최&gt; 22일 방미통위 '제24차 전체회의'를 열고 방송의 공적책임을 높이기 위한 안건들을 처리했습니다. 「전파법」을 위반한 (재)가톨릭평화방송에 대해 행정처분을 의결하고, 재허가·재승인을 받는 방송사업자의 '2024년도 방송에 대한 평가 결과'와 '2025년도 방송평가 더 보기</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://x.com/jkim386_kmcc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>방통위(김종철)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jkim386.kmcc)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21h</t>
+          <t>15시간</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 7월 27일 Hoje tive a honra de receber o presi</t>
+          <t>&lt; 디지털 플랫폼 이용자 권익 보호 &gt;… 더 보기</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jkim386.kmcc/posts/pfbid0m4fuHnjhMapvmsiQYMRkvbuh5XpXKuYJCcLLtVBSsfCGzb11NN4X1SVAFkZ37fWbl</t>
         </is>
       </c>
     </row>
@@ -625,12 +625,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>19h</t>
+          <t>55m</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 22h Hoje tive a honra de receber o presiden</t>
+          <t>남미 경제의 심장, 브라질 상파울루에서 양국의 미래를 함께 만들어 갈 기업인 여러분을 만났습니다. 브라질은 대한민국의 남미 최대 교역국이자 우리 기업들이 활발히 진출해 있는 나라입니다. 대한민국의 뛰어난 기술과 제조 역량이 브라질의 풍부한 자원, 성장 잠재력과 만난다면 양국은 더 보기</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -647,76 +647,76 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(jaemyunglee)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>53m</t>
+          <t>21시간</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Estimado Presidente José Antonio Kast. Chile es un país muy cercano e importante para la República de Corea, siendo el primer país con el que firmamos un Tratado de Libre Comercio (TLC). Espero con gran entusiasmo nuestra reunión. – Lee Jae-myung, Presidente de la República de 더 보기</t>
+          <t>&lt;지구 반대편 브라질에서 대한민국 경제와 외교의 지평을 넓혀갑니다&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://x.com/Jaemyung_Lee</t>
+          <t>https://www.facebook.com/jaemyunglee/posts/pfbid0CghEaiKD7bqfFgtRKuafzV8ScTiNNhYBbDEc281Z7pRb1xEfECLeeh3AnnqJUrVXl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대통령(이재명)</t>
+          <t>더불어민주당 대표(정청래)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>X(@Jaemyung_Lee)</t>
+          <t>Facebook(cheongrae1)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17h</t>
+          <t>1시간</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Agradeço em nome do povo sul-coreano pela calorosa recepção do Presidente Lula. @LulaOficial Vamos dar as mãos e, juntos, abrir um futuro novo e brilhante para os nossos países. 룰라 대통령님의 뜨거운 환대에 대한민국 국민을 대표하여 감사드립니다. 서로 손 맞잡고 양국의 새롭고 더 보기 Lula @LulaOficial 20h Hoje tive a honra de receber o presiden</t>
+          <t>&lt;여론은 추세가 중요하다.&gt;… 더 보기</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t